<commit_message>
Le PC veut redémarrer
</commit_message>
<xml_diff>
--- a/Doc/2_CAND_Modele_Planning_2026.xlsx
+++ b/Doc/2_CAND_Modele_Planning_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TPI - 2026 - Lucielle Voeffray\Dossier de projet\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B3EB737-B60E-485E-9B7D-A04DC3447DA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66E9AE26-945B-4998-AB76-1898E0919436}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1860" yWindow="1860" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planning EMF-EPAI" sheetId="8" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="64">
   <si>
     <t>Tâches</t>
   </si>
@@ -1160,7 +1160,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -1172,7 +1172,7 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -1184,7 +1184,7 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -1196,28 +1196,24 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" textRotation="90"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
@@ -1240,12 +1236,16 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" textRotation="90"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -1872,188 +1872,188 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:172" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A1" s="90" t="s">
+      <c r="A1" s="100" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
+      <c r="B1" s="100"/>
+      <c r="C1" s="100"/>
     </row>
     <row r="2" spans="1:172" ht="18" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B2" s="91">
+      <c r="B2" s="101">
         <v>157443</v>
       </c>
-      <c r="C2" s="92"/>
-      <c r="D2" s="99" t="s">
+      <c r="C2" s="102"/>
+      <c r="D2" s="98" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="99"/>
-      <c r="F2" s="99"/>
-      <c r="G2" s="99"/>
-      <c r="H2" s="99"/>
-      <c r="I2" s="99"/>
-      <c r="J2" s="99"/>
-      <c r="K2" s="99"/>
-      <c r="L2" s="99"/>
-      <c r="M2" s="99"/>
-      <c r="N2" s="99"/>
-      <c r="O2" s="99"/>
-      <c r="P2" s="99"/>
-      <c r="Q2" s="99"/>
-      <c r="R2" s="99"/>
-      <c r="S2" s="99"/>
-      <c r="T2" s="99"/>
-      <c r="U2" s="99"/>
-      <c r="V2" s="99"/>
-      <c r="W2" s="99"/>
-      <c r="X2" s="99"/>
-      <c r="Y2" s="99"/>
-      <c r="Z2" s="99"/>
-      <c r="AA2" s="99"/>
-      <c r="AB2" s="99"/>
-      <c r="AC2" s="99"/>
-      <c r="AD2" s="99"/>
-      <c r="AE2" s="99"/>
-      <c r="AF2" s="99"/>
-      <c r="AG2" s="99"/>
-      <c r="AH2" s="99"/>
-      <c r="AI2" s="99"/>
-      <c r="AJ2" s="99"/>
-      <c r="AK2" s="99"/>
-      <c r="AL2" s="99"/>
-      <c r="AM2" s="99"/>
-      <c r="AN2" s="99"/>
-      <c r="AO2" s="99"/>
-      <c r="AP2" s="99"/>
-      <c r="AQ2" s="99"/>
-      <c r="AR2" s="99" t="s">
+      <c r="E2" s="98"/>
+      <c r="F2" s="98"/>
+      <c r="G2" s="98"/>
+      <c r="H2" s="98"/>
+      <c r="I2" s="98"/>
+      <c r="J2" s="98"/>
+      <c r="K2" s="98"/>
+      <c r="L2" s="98"/>
+      <c r="M2" s="98"/>
+      <c r="N2" s="98"/>
+      <c r="O2" s="98"/>
+      <c r="P2" s="98"/>
+      <c r="Q2" s="98"/>
+      <c r="R2" s="98"/>
+      <c r="S2" s="98"/>
+      <c r="T2" s="98"/>
+      <c r="U2" s="98"/>
+      <c r="V2" s="98"/>
+      <c r="W2" s="98"/>
+      <c r="X2" s="98"/>
+      <c r="Y2" s="98"/>
+      <c r="Z2" s="98"/>
+      <c r="AA2" s="98"/>
+      <c r="AB2" s="98"/>
+      <c r="AC2" s="98"/>
+      <c r="AD2" s="98"/>
+      <c r="AE2" s="98"/>
+      <c r="AF2" s="98"/>
+      <c r="AG2" s="98"/>
+      <c r="AH2" s="98"/>
+      <c r="AI2" s="98"/>
+      <c r="AJ2" s="98"/>
+      <c r="AK2" s="98"/>
+      <c r="AL2" s="98"/>
+      <c r="AM2" s="98"/>
+      <c r="AN2" s="98"/>
+      <c r="AO2" s="98"/>
+      <c r="AP2" s="98"/>
+      <c r="AQ2" s="98"/>
+      <c r="AR2" s="98" t="s">
         <v>10</v>
       </c>
-      <c r="AS2" s="99"/>
-      <c r="AT2" s="99"/>
-      <c r="AU2" s="99"/>
-      <c r="AV2" s="99"/>
-      <c r="AW2" s="99"/>
-      <c r="AX2" s="99"/>
-      <c r="AY2" s="99"/>
-      <c r="AZ2" s="99"/>
-      <c r="BA2" s="99"/>
-      <c r="BB2" s="99"/>
-      <c r="BC2" s="99"/>
-      <c r="BD2" s="99"/>
-      <c r="BE2" s="99"/>
-      <c r="BF2" s="99"/>
-      <c r="BG2" s="99"/>
-      <c r="BH2" s="99"/>
-      <c r="BI2" s="99"/>
-      <c r="BJ2" s="99"/>
-      <c r="BK2" s="99"/>
-      <c r="BL2" s="99"/>
-      <c r="BM2" s="99"/>
-      <c r="BN2" s="99"/>
-      <c r="BO2" s="99"/>
-      <c r="BP2" s="99"/>
-      <c r="BQ2" s="99"/>
-      <c r="BR2" s="99"/>
-      <c r="BS2" s="99"/>
-      <c r="BT2" s="99"/>
-      <c r="BU2" s="99"/>
-      <c r="BV2" s="99"/>
-      <c r="BW2" s="99"/>
-      <c r="BX2" s="99"/>
-      <c r="BY2" s="99"/>
-      <c r="BZ2" s="99"/>
-      <c r="CA2" s="99"/>
-      <c r="CB2" s="99"/>
-      <c r="CC2" s="99"/>
-      <c r="CD2" s="99"/>
-      <c r="CE2" s="99"/>
-      <c r="CF2" s="99" t="s">
+      <c r="AS2" s="98"/>
+      <c r="AT2" s="98"/>
+      <c r="AU2" s="98"/>
+      <c r="AV2" s="98"/>
+      <c r="AW2" s="98"/>
+      <c r="AX2" s="98"/>
+      <c r="AY2" s="98"/>
+      <c r="AZ2" s="98"/>
+      <c r="BA2" s="98"/>
+      <c r="BB2" s="98"/>
+      <c r="BC2" s="98"/>
+      <c r="BD2" s="98"/>
+      <c r="BE2" s="98"/>
+      <c r="BF2" s="98"/>
+      <c r="BG2" s="98"/>
+      <c r="BH2" s="98"/>
+      <c r="BI2" s="98"/>
+      <c r="BJ2" s="98"/>
+      <c r="BK2" s="98"/>
+      <c r="BL2" s="98"/>
+      <c r="BM2" s="98"/>
+      <c r="BN2" s="98"/>
+      <c r="BO2" s="98"/>
+      <c r="BP2" s="98"/>
+      <c r="BQ2" s="98"/>
+      <c r="BR2" s="98"/>
+      <c r="BS2" s="98"/>
+      <c r="BT2" s="98"/>
+      <c r="BU2" s="98"/>
+      <c r="BV2" s="98"/>
+      <c r="BW2" s="98"/>
+      <c r="BX2" s="98"/>
+      <c r="BY2" s="98"/>
+      <c r="BZ2" s="98"/>
+      <c r="CA2" s="98"/>
+      <c r="CB2" s="98"/>
+      <c r="CC2" s="98"/>
+      <c r="CD2" s="98"/>
+      <c r="CE2" s="98"/>
+      <c r="CF2" s="98" t="s">
         <v>10</v>
       </c>
-      <c r="CG2" s="99"/>
-      <c r="CH2" s="99"/>
-      <c r="CI2" s="99"/>
-      <c r="CJ2" s="99"/>
-      <c r="CK2" s="99"/>
-      <c r="CL2" s="99"/>
-      <c r="CM2" s="99"/>
-      <c r="CN2" s="99"/>
-      <c r="CO2" s="99"/>
-      <c r="CP2" s="99"/>
-      <c r="CQ2" s="99"/>
-      <c r="CR2" s="99"/>
-      <c r="CS2" s="99"/>
-      <c r="CT2" s="99"/>
-      <c r="CU2" s="99"/>
-      <c r="CV2" s="99"/>
-      <c r="CW2" s="99"/>
-      <c r="CX2" s="99"/>
-      <c r="CY2" s="99"/>
-      <c r="CZ2" s="99"/>
-      <c r="DA2" s="99"/>
-      <c r="DB2" s="99"/>
-      <c r="DC2" s="99"/>
-      <c r="DD2" s="99"/>
-      <c r="DE2" s="99"/>
-      <c r="DF2" s="99"/>
-      <c r="DG2" s="99"/>
-      <c r="DH2" s="99"/>
-      <c r="DI2" s="99"/>
-      <c r="DJ2" s="99"/>
-      <c r="DK2" s="99"/>
-      <c r="DL2" s="99"/>
-      <c r="DM2" s="99"/>
-      <c r="DN2" s="99"/>
-      <c r="DO2" s="99"/>
-      <c r="DP2" s="99"/>
-      <c r="DQ2" s="99"/>
-      <c r="DR2" s="99"/>
-      <c r="DS2" s="99"/>
-      <c r="DT2" s="99" t="s">
+      <c r="CG2" s="98"/>
+      <c r="CH2" s="98"/>
+      <c r="CI2" s="98"/>
+      <c r="CJ2" s="98"/>
+      <c r="CK2" s="98"/>
+      <c r="CL2" s="98"/>
+      <c r="CM2" s="98"/>
+      <c r="CN2" s="98"/>
+      <c r="CO2" s="98"/>
+      <c r="CP2" s="98"/>
+      <c r="CQ2" s="98"/>
+      <c r="CR2" s="98"/>
+      <c r="CS2" s="98"/>
+      <c r="CT2" s="98"/>
+      <c r="CU2" s="98"/>
+      <c r="CV2" s="98"/>
+      <c r="CW2" s="98"/>
+      <c r="CX2" s="98"/>
+      <c r="CY2" s="98"/>
+      <c r="CZ2" s="98"/>
+      <c r="DA2" s="98"/>
+      <c r="DB2" s="98"/>
+      <c r="DC2" s="98"/>
+      <c r="DD2" s="98"/>
+      <c r="DE2" s="98"/>
+      <c r="DF2" s="98"/>
+      <c r="DG2" s="98"/>
+      <c r="DH2" s="98"/>
+      <c r="DI2" s="98"/>
+      <c r="DJ2" s="98"/>
+      <c r="DK2" s="98"/>
+      <c r="DL2" s="98"/>
+      <c r="DM2" s="98"/>
+      <c r="DN2" s="98"/>
+      <c r="DO2" s="98"/>
+      <c r="DP2" s="98"/>
+      <c r="DQ2" s="98"/>
+      <c r="DR2" s="98"/>
+      <c r="DS2" s="98"/>
+      <c r="DT2" s="98" t="s">
         <v>10</v>
       </c>
-      <c r="DU2" s="99"/>
-      <c r="DV2" s="99"/>
-      <c r="DW2" s="99"/>
-      <c r="DX2" s="99"/>
-      <c r="DY2" s="99"/>
-      <c r="DZ2" s="99"/>
-      <c r="EA2" s="99"/>
-      <c r="EB2" s="99"/>
-      <c r="EC2" s="99"/>
-      <c r="ED2" s="99"/>
-      <c r="EE2" s="99"/>
-      <c r="EF2" s="99"/>
-      <c r="EG2" s="99"/>
-      <c r="EH2" s="99"/>
-      <c r="EI2" s="99"/>
-      <c r="EJ2" s="99"/>
-      <c r="EK2" s="99"/>
-      <c r="EL2" s="99"/>
-      <c r="EM2" s="99"/>
-      <c r="EN2" s="99"/>
-      <c r="EO2" s="99"/>
-      <c r="EP2" s="99"/>
-      <c r="EQ2" s="99"/>
-      <c r="ER2" s="99"/>
-      <c r="ES2" s="99"/>
-      <c r="ET2" s="99"/>
-      <c r="EU2" s="99"/>
-      <c r="EV2" s="99"/>
-      <c r="EW2" s="99"/>
-      <c r="EX2" s="99"/>
-      <c r="EY2" s="99"/>
-      <c r="EZ2" s="99"/>
-      <c r="FA2" s="99"/>
-      <c r="FB2" s="99"/>
-      <c r="FC2" s="99"/>
-      <c r="FD2" s="99"/>
-      <c r="FE2" s="99"/>
-      <c r="FF2" s="99"/>
-      <c r="FG2" s="99"/>
+      <c r="DU2" s="98"/>
+      <c r="DV2" s="98"/>
+      <c r="DW2" s="98"/>
+      <c r="DX2" s="98"/>
+      <c r="DY2" s="98"/>
+      <c r="DZ2" s="98"/>
+      <c r="EA2" s="98"/>
+      <c r="EB2" s="98"/>
+      <c r="EC2" s="98"/>
+      <c r="ED2" s="98"/>
+      <c r="EE2" s="98"/>
+      <c r="EF2" s="98"/>
+      <c r="EG2" s="98"/>
+      <c r="EH2" s="98"/>
+      <c r="EI2" s="98"/>
+      <c r="EJ2" s="98"/>
+      <c r="EK2" s="98"/>
+      <c r="EL2" s="98"/>
+      <c r="EM2" s="98"/>
+      <c r="EN2" s="98"/>
+      <c r="EO2" s="98"/>
+      <c r="EP2" s="98"/>
+      <c r="EQ2" s="98"/>
+      <c r="ER2" s="98"/>
+      <c r="ES2" s="98"/>
+      <c r="ET2" s="98"/>
+      <c r="EU2" s="98"/>
+      <c r="EV2" s="98"/>
+      <c r="EW2" s="98"/>
+      <c r="EX2" s="98"/>
+      <c r="EY2" s="98"/>
+      <c r="EZ2" s="98"/>
+      <c r="FA2" s="98"/>
+      <c r="FB2" s="98"/>
+      <c r="FC2" s="98"/>
+      <c r="FD2" s="98"/>
+      <c r="FE2" s="98"/>
+      <c r="FF2" s="98"/>
+      <c r="FG2" s="98"/>
       <c r="FH2" s="39"/>
       <c r="FI2" s="39"/>
       <c r="FJ2" s="39"/>
@@ -2064,166 +2064,166 @@
       <c r="FO2" s="39"/>
     </row>
     <row r="3" spans="1:172" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D3" s="100"/>
-      <c r="E3" s="100"/>
-      <c r="F3" s="100"/>
-      <c r="G3" s="100"/>
-      <c r="H3" s="100"/>
-      <c r="I3" s="100"/>
-      <c r="J3" s="100"/>
-      <c r="K3" s="100"/>
-      <c r="L3" s="100"/>
-      <c r="M3" s="100"/>
-      <c r="N3" s="100"/>
-      <c r="O3" s="100"/>
-      <c r="P3" s="100"/>
-      <c r="Q3" s="100"/>
-      <c r="R3" s="100"/>
-      <c r="S3" s="100"/>
-      <c r="T3" s="100"/>
-      <c r="U3" s="100"/>
-      <c r="V3" s="100"/>
-      <c r="W3" s="100"/>
-      <c r="X3" s="100"/>
-      <c r="Y3" s="100"/>
-      <c r="Z3" s="100"/>
-      <c r="AA3" s="100"/>
-      <c r="AB3" s="100"/>
-      <c r="AC3" s="100"/>
-      <c r="AD3" s="100"/>
-      <c r="AE3" s="100"/>
-      <c r="AF3" s="100"/>
-      <c r="AG3" s="100"/>
-      <c r="AH3" s="100"/>
-      <c r="AI3" s="100"/>
-      <c r="AJ3" s="100"/>
-      <c r="AK3" s="100"/>
-      <c r="AL3" s="100"/>
-      <c r="AM3" s="100"/>
-      <c r="AN3" s="100"/>
-      <c r="AO3" s="100"/>
-      <c r="AP3" s="100"/>
-      <c r="AQ3" s="100"/>
-      <c r="AR3" s="100"/>
-      <c r="AS3" s="100"/>
-      <c r="AT3" s="100"/>
-      <c r="AU3" s="100"/>
-      <c r="AV3" s="100"/>
-      <c r="AW3" s="100"/>
-      <c r="AX3" s="100"/>
-      <c r="AY3" s="100"/>
-      <c r="AZ3" s="100"/>
-      <c r="BA3" s="100"/>
-      <c r="BB3" s="100"/>
-      <c r="BC3" s="100"/>
-      <c r="BD3" s="100"/>
-      <c r="BE3" s="100"/>
-      <c r="BF3" s="100"/>
-      <c r="BG3" s="100"/>
-      <c r="BH3" s="100"/>
-      <c r="BI3" s="100"/>
-      <c r="BJ3" s="100"/>
-      <c r="BK3" s="100"/>
-      <c r="BL3" s="100"/>
-      <c r="BM3" s="100"/>
-      <c r="BN3" s="100"/>
-      <c r="BO3" s="100"/>
-      <c r="BP3" s="100"/>
-      <c r="BQ3" s="100"/>
-      <c r="BR3" s="100"/>
-      <c r="BS3" s="100"/>
-      <c r="BT3" s="100"/>
-      <c r="BU3" s="100"/>
-      <c r="BV3" s="100"/>
-      <c r="BW3" s="100"/>
-      <c r="BX3" s="100"/>
-      <c r="BY3" s="100"/>
-      <c r="BZ3" s="100"/>
-      <c r="CA3" s="100"/>
-      <c r="CB3" s="100"/>
-      <c r="CC3" s="100"/>
-      <c r="CD3" s="100"/>
-      <c r="CE3" s="100"/>
-      <c r="CF3" s="100"/>
-      <c r="CG3" s="100"/>
-      <c r="CH3" s="100"/>
-      <c r="CI3" s="100"/>
-      <c r="CJ3" s="100"/>
-      <c r="CK3" s="100"/>
-      <c r="CL3" s="100"/>
-      <c r="CM3" s="100"/>
-      <c r="CN3" s="100"/>
-      <c r="CO3" s="100"/>
-      <c r="CP3" s="100"/>
-      <c r="CQ3" s="100"/>
-      <c r="CR3" s="100"/>
-      <c r="CS3" s="100"/>
-      <c r="CT3" s="100"/>
-      <c r="CU3" s="100"/>
-      <c r="CV3" s="100"/>
-      <c r="CW3" s="100"/>
-      <c r="CX3" s="100"/>
-      <c r="CY3" s="100"/>
-      <c r="CZ3" s="100"/>
-      <c r="DA3" s="100"/>
-      <c r="DB3" s="100"/>
-      <c r="DC3" s="100"/>
-      <c r="DD3" s="100"/>
-      <c r="DE3" s="100"/>
-      <c r="DF3" s="100"/>
-      <c r="DG3" s="100"/>
-      <c r="DH3" s="100"/>
-      <c r="DI3" s="100"/>
-      <c r="DJ3" s="100"/>
-      <c r="DK3" s="100"/>
-      <c r="DL3" s="100"/>
-      <c r="DM3" s="100"/>
-      <c r="DN3" s="100"/>
-      <c r="DO3" s="100"/>
-      <c r="DP3" s="100"/>
-      <c r="DQ3" s="100"/>
-      <c r="DR3" s="100"/>
-      <c r="DS3" s="100"/>
-      <c r="DT3" s="100"/>
-      <c r="DU3" s="100"/>
-      <c r="DV3" s="100"/>
-      <c r="DW3" s="100"/>
-      <c r="DX3" s="100"/>
-      <c r="DY3" s="100"/>
-      <c r="DZ3" s="100"/>
-      <c r="EA3" s="100"/>
-      <c r="EB3" s="100"/>
-      <c r="EC3" s="100"/>
-      <c r="ED3" s="100"/>
-      <c r="EE3" s="100"/>
-      <c r="EF3" s="100"/>
-      <c r="EG3" s="100"/>
-      <c r="EH3" s="100"/>
-      <c r="EI3" s="100"/>
-      <c r="EJ3" s="100"/>
-      <c r="EK3" s="100"/>
-      <c r="EL3" s="100"/>
-      <c r="EM3" s="100"/>
-      <c r="EN3" s="100"/>
-      <c r="EO3" s="100"/>
-      <c r="EP3" s="100"/>
-      <c r="EQ3" s="100"/>
-      <c r="ER3" s="100"/>
-      <c r="ES3" s="100"/>
-      <c r="ET3" s="100"/>
-      <c r="EU3" s="100"/>
-      <c r="EV3" s="100"/>
-      <c r="EW3" s="100"/>
-      <c r="EX3" s="100"/>
-      <c r="EY3" s="100"/>
-      <c r="EZ3" s="100"/>
-      <c r="FA3" s="100"/>
-      <c r="FB3" s="100"/>
-      <c r="FC3" s="100"/>
-      <c r="FD3" s="100"/>
-      <c r="FE3" s="100"/>
-      <c r="FF3" s="100"/>
-      <c r="FG3" s="100"/>
+      <c r="D3" s="99"/>
+      <c r="E3" s="99"/>
+      <c r="F3" s="99"/>
+      <c r="G3" s="99"/>
+      <c r="H3" s="99"/>
+      <c r="I3" s="99"/>
+      <c r="J3" s="99"/>
+      <c r="K3" s="99"/>
+      <c r="L3" s="99"/>
+      <c r="M3" s="99"/>
+      <c r="N3" s="99"/>
+      <c r="O3" s="99"/>
+      <c r="P3" s="99"/>
+      <c r="Q3" s="99"/>
+      <c r="R3" s="99"/>
+      <c r="S3" s="99"/>
+      <c r="T3" s="99"/>
+      <c r="U3" s="99"/>
+      <c r="V3" s="99"/>
+      <c r="W3" s="99"/>
+      <c r="X3" s="99"/>
+      <c r="Y3" s="99"/>
+      <c r="Z3" s="99"/>
+      <c r="AA3" s="99"/>
+      <c r="AB3" s="99"/>
+      <c r="AC3" s="99"/>
+      <c r="AD3" s="99"/>
+      <c r="AE3" s="99"/>
+      <c r="AF3" s="99"/>
+      <c r="AG3" s="99"/>
+      <c r="AH3" s="99"/>
+      <c r="AI3" s="99"/>
+      <c r="AJ3" s="99"/>
+      <c r="AK3" s="99"/>
+      <c r="AL3" s="99"/>
+      <c r="AM3" s="99"/>
+      <c r="AN3" s="99"/>
+      <c r="AO3" s="99"/>
+      <c r="AP3" s="99"/>
+      <c r="AQ3" s="99"/>
+      <c r="AR3" s="99"/>
+      <c r="AS3" s="99"/>
+      <c r="AT3" s="99"/>
+      <c r="AU3" s="99"/>
+      <c r="AV3" s="99"/>
+      <c r="AW3" s="99"/>
+      <c r="AX3" s="99"/>
+      <c r="AY3" s="99"/>
+      <c r="AZ3" s="99"/>
+      <c r="BA3" s="99"/>
+      <c r="BB3" s="99"/>
+      <c r="BC3" s="99"/>
+      <c r="BD3" s="99"/>
+      <c r="BE3" s="99"/>
+      <c r="BF3" s="99"/>
+      <c r="BG3" s="99"/>
+      <c r="BH3" s="99"/>
+      <c r="BI3" s="99"/>
+      <c r="BJ3" s="99"/>
+      <c r="BK3" s="99"/>
+      <c r="BL3" s="99"/>
+      <c r="BM3" s="99"/>
+      <c r="BN3" s="99"/>
+      <c r="BO3" s="99"/>
+      <c r="BP3" s="99"/>
+      <c r="BQ3" s="99"/>
+      <c r="BR3" s="99"/>
+      <c r="BS3" s="99"/>
+      <c r="BT3" s="99"/>
+      <c r="BU3" s="99"/>
+      <c r="BV3" s="99"/>
+      <c r="BW3" s="99"/>
+      <c r="BX3" s="99"/>
+      <c r="BY3" s="99"/>
+      <c r="BZ3" s="99"/>
+      <c r="CA3" s="99"/>
+      <c r="CB3" s="99"/>
+      <c r="CC3" s="99"/>
+      <c r="CD3" s="99"/>
+      <c r="CE3" s="99"/>
+      <c r="CF3" s="99"/>
+      <c r="CG3" s="99"/>
+      <c r="CH3" s="99"/>
+      <c r="CI3" s="99"/>
+      <c r="CJ3" s="99"/>
+      <c r="CK3" s="99"/>
+      <c r="CL3" s="99"/>
+      <c r="CM3" s="99"/>
+      <c r="CN3" s="99"/>
+      <c r="CO3" s="99"/>
+      <c r="CP3" s="99"/>
+      <c r="CQ3" s="99"/>
+      <c r="CR3" s="99"/>
+      <c r="CS3" s="99"/>
+      <c r="CT3" s="99"/>
+      <c r="CU3" s="99"/>
+      <c r="CV3" s="99"/>
+      <c r="CW3" s="99"/>
+      <c r="CX3" s="99"/>
+      <c r="CY3" s="99"/>
+      <c r="CZ3" s="99"/>
+      <c r="DA3" s="99"/>
+      <c r="DB3" s="99"/>
+      <c r="DC3" s="99"/>
+      <c r="DD3" s="99"/>
+      <c r="DE3" s="99"/>
+      <c r="DF3" s="99"/>
+      <c r="DG3" s="99"/>
+      <c r="DH3" s="99"/>
+      <c r="DI3" s="99"/>
+      <c r="DJ3" s="99"/>
+      <c r="DK3" s="99"/>
+      <c r="DL3" s="99"/>
+      <c r="DM3" s="99"/>
+      <c r="DN3" s="99"/>
+      <c r="DO3" s="99"/>
+      <c r="DP3" s="99"/>
+      <c r="DQ3" s="99"/>
+      <c r="DR3" s="99"/>
+      <c r="DS3" s="99"/>
+      <c r="DT3" s="99"/>
+      <c r="DU3" s="99"/>
+      <c r="DV3" s="99"/>
+      <c r="DW3" s="99"/>
+      <c r="DX3" s="99"/>
+      <c r="DY3" s="99"/>
+      <c r="DZ3" s="99"/>
+      <c r="EA3" s="99"/>
+      <c r="EB3" s="99"/>
+      <c r="EC3" s="99"/>
+      <c r="ED3" s="99"/>
+      <c r="EE3" s="99"/>
+      <c r="EF3" s="99"/>
+      <c r="EG3" s="99"/>
+      <c r="EH3" s="99"/>
+      <c r="EI3" s="99"/>
+      <c r="EJ3" s="99"/>
+      <c r="EK3" s="99"/>
+      <c r="EL3" s="99"/>
+      <c r="EM3" s="99"/>
+      <c r="EN3" s="99"/>
+      <c r="EO3" s="99"/>
+      <c r="EP3" s="99"/>
+      <c r="EQ3" s="99"/>
+      <c r="ER3" s="99"/>
+      <c r="ES3" s="99"/>
+      <c r="ET3" s="99"/>
+      <c r="EU3" s="99"/>
+      <c r="EV3" s="99"/>
+      <c r="EW3" s="99"/>
+      <c r="EX3" s="99"/>
+      <c r="EY3" s="99"/>
+      <c r="EZ3" s="99"/>
+      <c r="FA3" s="99"/>
+      <c r="FB3" s="99"/>
+      <c r="FC3" s="99"/>
+      <c r="FD3" s="99"/>
+      <c r="FE3" s="99"/>
+      <c r="FF3" s="99"/>
+      <c r="FG3" s="99"/>
       <c r="FH3" s="39"/>
       <c r="FI3" s="39"/>
       <c r="FJ3" s="39"/>
@@ -2234,7 +2234,7 @@
       <c r="FO3" s="39"/>
     </row>
     <row r="4" spans="1:172" x14ac:dyDescent="0.2">
-      <c r="A4" s="97" t="s">
+      <c r="A4" s="96" t="s">
         <v>0</v>
       </c>
       <c r="B4" s="25" t="s">
@@ -2495,12 +2495,12 @@
       <c r="FM4" s="68"/>
       <c r="FN4" s="68"/>
       <c r="FO4" s="69"/>
-      <c r="FP4" s="101" t="s">
+      <c r="FP4" s="94" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:172" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="98"/>
+      <c r="A5" s="97"/>
       <c r="B5" s="26" t="s">
         <v>3</v>
       </c>
@@ -3011,7 +3011,7 @@
       <c r="FO5" s="6">
         <v>8</v>
       </c>
-      <c r="FP5" s="101"/>
+      <c r="FP5" s="94"/>
     </row>
     <row r="6" spans="1:172" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="29" t="s">
@@ -3033,13 +3033,13 @@
       <c r="M6" s="9"/>
       <c r="N6" s="9"/>
       <c r="O6" s="9"/>
-      <c r="P6" s="93" t="s">
+      <c r="P6" s="81" t="s">
         <v>32</v>
       </c>
       <c r="Q6" s="82"/>
       <c r="R6" s="82"/>
       <c r="S6" s="83"/>
-      <c r="T6" s="81" t="s">
+      <c r="T6" s="90" t="s">
         <v>32</v>
       </c>
       <c r="U6" s="82"/>
@@ -3079,13 +3079,13 @@
       <c r="BA6" s="9"/>
       <c r="BB6" s="9"/>
       <c r="BC6" s="9"/>
-      <c r="BD6" s="93" t="s">
+      <c r="BD6" s="81" t="s">
         <v>32</v>
       </c>
       <c r="BE6" s="82"/>
       <c r="BF6" s="82"/>
       <c r="BG6" s="83"/>
-      <c r="BH6" s="81" t="s">
+      <c r="BH6" s="90" t="s">
         <v>32</v>
       </c>
       <c r="BI6" s="82"/>
@@ -3095,7 +3095,7 @@
       <c r="BM6" s="82"/>
       <c r="BN6" s="82"/>
       <c r="BO6" s="83"/>
-      <c r="BP6" s="93" t="s">
+      <c r="BP6" s="81" t="s">
         <v>32</v>
       </c>
       <c r="BQ6" s="82"/>
@@ -3123,7 +3123,7 @@
       <c r="CK6" s="73"/>
       <c r="CL6" s="73"/>
       <c r="CM6" s="74"/>
-      <c r="CN6" s="102" t="s">
+      <c r="CN6" s="93" t="s">
         <v>62</v>
       </c>
       <c r="CO6" s="82"/>
@@ -3169,13 +3169,13 @@
       <c r="EC6" s="9"/>
       <c r="ED6" s="9"/>
       <c r="EE6" s="9"/>
-      <c r="EF6" s="93" t="s">
+      <c r="EF6" s="81" t="s">
         <v>32</v>
       </c>
       <c r="EG6" s="82"/>
       <c r="EH6" s="82"/>
       <c r="EI6" s="83"/>
-      <c r="EJ6" s="81" t="s">
+      <c r="EJ6" s="90" t="s">
         <v>32</v>
       </c>
       <c r="EK6" s="82"/>
@@ -3211,7 +3211,7 @@
       <c r="FM6" s="9"/>
       <c r="FN6" s="9"/>
       <c r="FO6" s="9"/>
-      <c r="FP6" s="101"/>
+      <c r="FP6" s="94"/>
     </row>
     <row r="7" spans="1:172" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -3235,11 +3235,11 @@
       <c r="M7" s="15"/>
       <c r="N7" s="15"/>
       <c r="O7" s="15"/>
-      <c r="P7" s="94"/>
+      <c r="P7" s="84"/>
       <c r="Q7" s="85"/>
       <c r="R7" s="85"/>
       <c r="S7" s="86"/>
-      <c r="T7" s="84"/>
+      <c r="T7" s="91"/>
       <c r="U7" s="85"/>
       <c r="V7" s="85"/>
       <c r="W7" s="85"/>
@@ -3275,11 +3275,11 @@
       <c r="BA7" s="15"/>
       <c r="BB7" s="15"/>
       <c r="BC7" s="15"/>
-      <c r="BD7" s="94"/>
+      <c r="BD7" s="84"/>
       <c r="BE7" s="85"/>
       <c r="BF7" s="85"/>
       <c r="BG7" s="86"/>
-      <c r="BH7" s="84"/>
+      <c r="BH7" s="91"/>
       <c r="BI7" s="85"/>
       <c r="BJ7" s="85"/>
       <c r="BK7" s="85"/>
@@ -3287,7 +3287,7 @@
       <c r="BM7" s="85"/>
       <c r="BN7" s="85"/>
       <c r="BO7" s="86"/>
-      <c r="BP7" s="94"/>
+      <c r="BP7" s="84"/>
       <c r="BQ7" s="85"/>
       <c r="BR7" s="85"/>
       <c r="BS7" s="86"/>
@@ -3311,7 +3311,7 @@
       <c r="CK7" s="76"/>
       <c r="CL7" s="76"/>
       <c r="CM7" s="77"/>
-      <c r="CN7" s="84"/>
+      <c r="CN7" s="91"/>
       <c r="CO7" s="85"/>
       <c r="CP7" s="85"/>
       <c r="CQ7" s="85"/>
@@ -3355,11 +3355,11 @@
       <c r="EC7" s="15"/>
       <c r="ED7" s="15"/>
       <c r="EE7" s="15"/>
-      <c r="EF7" s="94"/>
+      <c r="EF7" s="84"/>
       <c r="EG7" s="85"/>
       <c r="EH7" s="85"/>
       <c r="EI7" s="86"/>
-      <c r="EJ7" s="84"/>
+      <c r="EJ7" s="91"/>
       <c r="EK7" s="85"/>
       <c r="EL7" s="85"/>
       <c r="EM7" s="85"/>
@@ -3391,7 +3391,7 @@
       <c r="FM7" s="15"/>
       <c r="FN7" s="15"/>
       <c r="FO7" s="15"/>
-      <c r="FP7" s="101"/>
+      <c r="FP7" s="94"/>
     </row>
     <row r="8" spans="1:172" x14ac:dyDescent="0.2">
       <c r="A8" s="12" t="s">
@@ -3415,11 +3415,11 @@
       <c r="M8" s="15"/>
       <c r="N8" s="15"/>
       <c r="O8" s="15"/>
-      <c r="P8" s="94"/>
+      <c r="P8" s="84"/>
       <c r="Q8" s="85"/>
       <c r="R8" s="85"/>
       <c r="S8" s="86"/>
-      <c r="T8" s="84"/>
+      <c r="T8" s="91"/>
       <c r="U8" s="85"/>
       <c r="V8" s="85"/>
       <c r="W8" s="85"/>
@@ -3455,11 +3455,11 @@
       <c r="BA8" s="15"/>
       <c r="BB8" s="15"/>
       <c r="BC8" s="15"/>
-      <c r="BD8" s="94"/>
+      <c r="BD8" s="84"/>
       <c r="BE8" s="85"/>
       <c r="BF8" s="85"/>
       <c r="BG8" s="86"/>
-      <c r="BH8" s="84"/>
+      <c r="BH8" s="91"/>
       <c r="BI8" s="85"/>
       <c r="BJ8" s="85"/>
       <c r="BK8" s="85"/>
@@ -3467,7 +3467,7 @@
       <c r="BM8" s="85"/>
       <c r="BN8" s="85"/>
       <c r="BO8" s="86"/>
-      <c r="BP8" s="94"/>
+      <c r="BP8" s="84"/>
       <c r="BQ8" s="85"/>
       <c r="BR8" s="85"/>
       <c r="BS8" s="86"/>
@@ -3491,7 +3491,7 @@
       <c r="CK8" s="76"/>
       <c r="CL8" s="76"/>
       <c r="CM8" s="77"/>
-      <c r="CN8" s="84"/>
+      <c r="CN8" s="91"/>
       <c r="CO8" s="85"/>
       <c r="CP8" s="85"/>
       <c r="CQ8" s="85"/>
@@ -3535,11 +3535,11 @@
       <c r="EC8" s="15"/>
       <c r="ED8" s="15"/>
       <c r="EE8" s="15"/>
-      <c r="EF8" s="94"/>
+      <c r="EF8" s="84"/>
       <c r="EG8" s="85"/>
       <c r="EH8" s="85"/>
       <c r="EI8" s="86"/>
-      <c r="EJ8" s="84"/>
+      <c r="EJ8" s="91"/>
       <c r="EK8" s="85"/>
       <c r="EL8" s="85"/>
       <c r="EM8" s="85"/>
@@ -3571,7 +3571,7 @@
       <c r="FM8" s="15"/>
       <c r="FN8" s="15"/>
       <c r="FO8" s="15"/>
-      <c r="FP8" s="101"/>
+      <c r="FP8" s="94"/>
     </row>
     <row r="9" spans="1:172" x14ac:dyDescent="0.2">
       <c r="A9" s="12" t="s">
@@ -3597,11 +3597,11 @@
       <c r="M9" s="15"/>
       <c r="N9" s="15"/>
       <c r="O9" s="15"/>
-      <c r="P9" s="94"/>
+      <c r="P9" s="84"/>
       <c r="Q9" s="85"/>
       <c r="R9" s="85"/>
       <c r="S9" s="86"/>
-      <c r="T9" s="84"/>
+      <c r="T9" s="91"/>
       <c r="U9" s="85"/>
       <c r="V9" s="85"/>
       <c r="W9" s="85"/>
@@ -3637,11 +3637,11 @@
       <c r="BA9" s="15"/>
       <c r="BB9" s="15"/>
       <c r="BC9" s="15"/>
-      <c r="BD9" s="94"/>
+      <c r="BD9" s="84"/>
       <c r="BE9" s="85"/>
       <c r="BF9" s="85"/>
       <c r="BG9" s="86"/>
-      <c r="BH9" s="84"/>
+      <c r="BH9" s="91"/>
       <c r="BI9" s="85"/>
       <c r="BJ9" s="85"/>
       <c r="BK9" s="85"/>
@@ -3649,7 +3649,7 @@
       <c r="BM9" s="85"/>
       <c r="BN9" s="85"/>
       <c r="BO9" s="86"/>
-      <c r="BP9" s="94"/>
+      <c r="BP9" s="84"/>
       <c r="BQ9" s="85"/>
       <c r="BR9" s="85"/>
       <c r="BS9" s="86"/>
@@ -3673,7 +3673,7 @@
       <c r="CK9" s="76"/>
       <c r="CL9" s="76"/>
       <c r="CM9" s="77"/>
-      <c r="CN9" s="84"/>
+      <c r="CN9" s="91"/>
       <c r="CO9" s="85"/>
       <c r="CP9" s="85"/>
       <c r="CQ9" s="85"/>
@@ -3717,11 +3717,11 @@
       <c r="EC9" s="15"/>
       <c r="ED9" s="15"/>
       <c r="EE9" s="15"/>
-      <c r="EF9" s="94"/>
+      <c r="EF9" s="84"/>
       <c r="EG9" s="85"/>
       <c r="EH9" s="85"/>
       <c r="EI9" s="86"/>
-      <c r="EJ9" s="84"/>
+      <c r="EJ9" s="91"/>
       <c r="EK9" s="85"/>
       <c r="EL9" s="85"/>
       <c r="EM9" s="85"/>
@@ -3753,7 +3753,7 @@
       <c r="FM9" s="15"/>
       <c r="FN9" s="15"/>
       <c r="FO9" s="15"/>
-      <c r="FP9" s="101"/>
+      <c r="FP9" s="94"/>
     </row>
     <row r="10" spans="1:172" x14ac:dyDescent="0.2">
       <c r="A10" s="12" t="s">
@@ -3777,11 +3777,11 @@
       <c r="M10" s="15"/>
       <c r="N10" s="15"/>
       <c r="O10" s="15"/>
-      <c r="P10" s="94"/>
+      <c r="P10" s="84"/>
       <c r="Q10" s="85"/>
       <c r="R10" s="85"/>
       <c r="S10" s="86"/>
-      <c r="T10" s="84"/>
+      <c r="T10" s="91"/>
       <c r="U10" s="85"/>
       <c r="V10" s="85"/>
       <c r="W10" s="85"/>
@@ -3817,11 +3817,11 @@
       <c r="BA10" s="15"/>
       <c r="BB10" s="15"/>
       <c r="BC10" s="15"/>
-      <c r="BD10" s="94"/>
+      <c r="BD10" s="84"/>
       <c r="BE10" s="85"/>
       <c r="BF10" s="85"/>
       <c r="BG10" s="86"/>
-      <c r="BH10" s="84"/>
+      <c r="BH10" s="91"/>
       <c r="BI10" s="85"/>
       <c r="BJ10" s="85"/>
       <c r="BK10" s="85"/>
@@ -3829,7 +3829,7 @@
       <c r="BM10" s="85"/>
       <c r="BN10" s="85"/>
       <c r="BO10" s="86"/>
-      <c r="BP10" s="94"/>
+      <c r="BP10" s="84"/>
       <c r="BQ10" s="85"/>
       <c r="BR10" s="85"/>
       <c r="BS10" s="86"/>
@@ -3853,7 +3853,7 @@
       <c r="CK10" s="76"/>
       <c r="CL10" s="76"/>
       <c r="CM10" s="77"/>
-      <c r="CN10" s="84"/>
+      <c r="CN10" s="91"/>
       <c r="CO10" s="85"/>
       <c r="CP10" s="85"/>
       <c r="CQ10" s="85"/>
@@ -3897,11 +3897,11 @@
       <c r="EC10" s="15"/>
       <c r="ED10" s="15"/>
       <c r="EE10" s="15"/>
-      <c r="EF10" s="94"/>
+      <c r="EF10" s="84"/>
       <c r="EG10" s="85"/>
       <c r="EH10" s="85"/>
       <c r="EI10" s="86"/>
-      <c r="EJ10" s="84"/>
+      <c r="EJ10" s="91"/>
       <c r="EK10" s="85"/>
       <c r="EL10" s="85"/>
       <c r="EM10" s="85"/>
@@ -3933,7 +3933,7 @@
       <c r="FM10" s="15"/>
       <c r="FN10" s="15"/>
       <c r="FO10" s="15"/>
-      <c r="FP10" s="101"/>
+      <c r="FP10" s="94"/>
     </row>
     <row r="11" spans="1:172" x14ac:dyDescent="0.2">
       <c r="A11" s="12" t="s">
@@ -3957,11 +3957,11 @@
       <c r="M11" s="15"/>
       <c r="N11" s="15"/>
       <c r="O11" s="15"/>
-      <c r="P11" s="94"/>
+      <c r="P11" s="84"/>
       <c r="Q11" s="85"/>
       <c r="R11" s="85"/>
       <c r="S11" s="86"/>
-      <c r="T11" s="84"/>
+      <c r="T11" s="91"/>
       <c r="U11" s="85"/>
       <c r="V11" s="85"/>
       <c r="W11" s="85"/>
@@ -3997,11 +3997,11 @@
       <c r="BA11" s="15"/>
       <c r="BB11" s="15"/>
       <c r="BC11" s="15"/>
-      <c r="BD11" s="94"/>
+      <c r="BD11" s="84"/>
       <c r="BE11" s="85"/>
       <c r="BF11" s="85"/>
       <c r="BG11" s="86"/>
-      <c r="BH11" s="84"/>
+      <c r="BH11" s="91"/>
       <c r="BI11" s="85"/>
       <c r="BJ11" s="85"/>
       <c r="BK11" s="85"/>
@@ -4009,7 +4009,7 @@
       <c r="BM11" s="85"/>
       <c r="BN11" s="85"/>
       <c r="BO11" s="86"/>
-      <c r="BP11" s="94"/>
+      <c r="BP11" s="84"/>
       <c r="BQ11" s="85"/>
       <c r="BR11" s="85"/>
       <c r="BS11" s="86"/>
@@ -4033,7 +4033,7 @@
       <c r="CK11" s="76"/>
       <c r="CL11" s="76"/>
       <c r="CM11" s="77"/>
-      <c r="CN11" s="84"/>
+      <c r="CN11" s="91"/>
       <c r="CO11" s="85"/>
       <c r="CP11" s="85"/>
       <c r="CQ11" s="85"/>
@@ -4077,11 +4077,11 @@
       <c r="EC11" s="15"/>
       <c r="ED11" s="15"/>
       <c r="EE11" s="15"/>
-      <c r="EF11" s="94"/>
+      <c r="EF11" s="84"/>
       <c r="EG11" s="85"/>
       <c r="EH11" s="85"/>
       <c r="EI11" s="86"/>
-      <c r="EJ11" s="84"/>
+      <c r="EJ11" s="91"/>
       <c r="EK11" s="85"/>
       <c r="EL11" s="85"/>
       <c r="EM11" s="85"/>
@@ -4113,7 +4113,7 @@
       <c r="FM11" s="15"/>
       <c r="FN11" s="15"/>
       <c r="FO11" s="15"/>
-      <c r="FP11" s="101"/>
+      <c r="FP11" s="94"/>
     </row>
     <row r="12" spans="1:172" x14ac:dyDescent="0.2">
       <c r="A12" s="12" t="s">
@@ -4136,11 +4136,11 @@
       <c r="M12" s="15"/>
       <c r="N12" s="15"/>
       <c r="O12" s="15"/>
-      <c r="P12" s="94"/>
+      <c r="P12" s="84"/>
       <c r="Q12" s="85"/>
       <c r="R12" s="85"/>
       <c r="S12" s="86"/>
-      <c r="T12" s="84"/>
+      <c r="T12" s="91"/>
       <c r="U12" s="85"/>
       <c r="V12" s="85"/>
       <c r="W12" s="85"/>
@@ -4176,11 +4176,11 @@
       <c r="BA12" s="15"/>
       <c r="BB12" s="15"/>
       <c r="BC12" s="15"/>
-      <c r="BD12" s="94"/>
+      <c r="BD12" s="84"/>
       <c r="BE12" s="85"/>
       <c r="BF12" s="85"/>
       <c r="BG12" s="86"/>
-      <c r="BH12" s="84"/>
+      <c r="BH12" s="91"/>
       <c r="BI12" s="85"/>
       <c r="BJ12" s="85"/>
       <c r="BK12" s="85"/>
@@ -4188,7 +4188,7 @@
       <c r="BM12" s="85"/>
       <c r="BN12" s="85"/>
       <c r="BO12" s="86"/>
-      <c r="BP12" s="94"/>
+      <c r="BP12" s="84"/>
       <c r="BQ12" s="85"/>
       <c r="BR12" s="85"/>
       <c r="BS12" s="86"/>
@@ -4212,7 +4212,7 @@
       <c r="CK12" s="76"/>
       <c r="CL12" s="76"/>
       <c r="CM12" s="77"/>
-      <c r="CN12" s="84"/>
+      <c r="CN12" s="91"/>
       <c r="CO12" s="85"/>
       <c r="CP12" s="85"/>
       <c r="CQ12" s="85"/>
@@ -4256,11 +4256,11 @@
       <c r="EC12" s="15"/>
       <c r="ED12" s="15"/>
       <c r="EE12" s="15"/>
-      <c r="EF12" s="94"/>
+      <c r="EF12" s="84"/>
       <c r="EG12" s="85"/>
       <c r="EH12" s="85"/>
       <c r="EI12" s="86"/>
-      <c r="EJ12" s="84"/>
+      <c r="EJ12" s="91"/>
       <c r="EK12" s="85"/>
       <c r="EL12" s="85"/>
       <c r="EM12" s="85"/>
@@ -4292,7 +4292,7 @@
       <c r="FM12" s="15"/>
       <c r="FN12" s="15"/>
       <c r="FO12" s="15"/>
-      <c r="FP12" s="101"/>
+      <c r="FP12" s="94"/>
     </row>
     <row r="13" spans="1:172" x14ac:dyDescent="0.2">
       <c r="A13" s="12" t="s">
@@ -4316,11 +4316,11 @@
       <c r="M13" s="15"/>
       <c r="N13" s="15"/>
       <c r="O13" s="15"/>
-      <c r="P13" s="94"/>
+      <c r="P13" s="84"/>
       <c r="Q13" s="85"/>
       <c r="R13" s="85"/>
       <c r="S13" s="86"/>
-      <c r="T13" s="84"/>
+      <c r="T13" s="91"/>
       <c r="U13" s="85"/>
       <c r="V13" s="85"/>
       <c r="W13" s="85"/>
@@ -4356,11 +4356,11 @@
       <c r="BA13" s="15"/>
       <c r="BB13" s="15"/>
       <c r="BC13" s="15"/>
-      <c r="BD13" s="94"/>
+      <c r="BD13" s="84"/>
       <c r="BE13" s="85"/>
       <c r="BF13" s="85"/>
       <c r="BG13" s="86"/>
-      <c r="BH13" s="84"/>
+      <c r="BH13" s="91"/>
       <c r="BI13" s="85"/>
       <c r="BJ13" s="85"/>
       <c r="BK13" s="85"/>
@@ -4368,7 +4368,7 @@
       <c r="BM13" s="85"/>
       <c r="BN13" s="85"/>
       <c r="BO13" s="86"/>
-      <c r="BP13" s="94"/>
+      <c r="BP13" s="84"/>
       <c r="BQ13" s="85"/>
       <c r="BR13" s="85"/>
       <c r="BS13" s="86"/>
@@ -4392,7 +4392,7 @@
       <c r="CK13" s="76"/>
       <c r="CL13" s="76"/>
       <c r="CM13" s="77"/>
-      <c r="CN13" s="84"/>
+      <c r="CN13" s="91"/>
       <c r="CO13" s="85"/>
       <c r="CP13" s="85"/>
       <c r="CQ13" s="85"/>
@@ -4436,11 +4436,11 @@
       <c r="EC13" s="15"/>
       <c r="ED13" s="15"/>
       <c r="EE13" s="15"/>
-      <c r="EF13" s="94"/>
+      <c r="EF13" s="84"/>
       <c r="EG13" s="85"/>
       <c r="EH13" s="85"/>
       <c r="EI13" s="86"/>
-      <c r="EJ13" s="84"/>
+      <c r="EJ13" s="91"/>
       <c r="EK13" s="85"/>
       <c r="EL13" s="85"/>
       <c r="EM13" s="85"/>
@@ -4472,7 +4472,7 @@
       <c r="FM13" s="15"/>
       <c r="FN13" s="15"/>
       <c r="FO13" s="15"/>
-      <c r="FP13" s="101"/>
+      <c r="FP13" s="94"/>
     </row>
     <row r="14" spans="1:172" x14ac:dyDescent="0.2">
       <c r="A14" s="12"/>
@@ -4490,11 +4490,11 @@
       <c r="M14" s="15"/>
       <c r="N14" s="15"/>
       <c r="O14" s="15"/>
-      <c r="P14" s="94"/>
+      <c r="P14" s="84"/>
       <c r="Q14" s="85"/>
       <c r="R14" s="85"/>
       <c r="S14" s="86"/>
-      <c r="T14" s="84"/>
+      <c r="T14" s="91"/>
       <c r="U14" s="85"/>
       <c r="V14" s="85"/>
       <c r="W14" s="85"/>
@@ -4530,11 +4530,11 @@
       <c r="BA14" s="15"/>
       <c r="BB14" s="15"/>
       <c r="BC14" s="15"/>
-      <c r="BD14" s="94"/>
+      <c r="BD14" s="84"/>
       <c r="BE14" s="85"/>
       <c r="BF14" s="85"/>
       <c r="BG14" s="86"/>
-      <c r="BH14" s="84"/>
+      <c r="BH14" s="91"/>
       <c r="BI14" s="85"/>
       <c r="BJ14" s="85"/>
       <c r="BK14" s="85"/>
@@ -4542,7 +4542,7 @@
       <c r="BM14" s="85"/>
       <c r="BN14" s="85"/>
       <c r="BO14" s="86"/>
-      <c r="BP14" s="94"/>
+      <c r="BP14" s="84"/>
       <c r="BQ14" s="85"/>
       <c r="BR14" s="85"/>
       <c r="BS14" s="86"/>
@@ -4566,7 +4566,7 @@
       <c r="CK14" s="76"/>
       <c r="CL14" s="76"/>
       <c r="CM14" s="77"/>
-      <c r="CN14" s="84"/>
+      <c r="CN14" s="91"/>
       <c r="CO14" s="85"/>
       <c r="CP14" s="85"/>
       <c r="CQ14" s="85"/>
@@ -4610,11 +4610,11 @@
       <c r="EC14" s="15"/>
       <c r="ED14" s="15"/>
       <c r="EE14" s="15"/>
-      <c r="EF14" s="94"/>
+      <c r="EF14" s="84"/>
       <c r="EG14" s="85"/>
       <c r="EH14" s="85"/>
       <c r="EI14" s="86"/>
-      <c r="EJ14" s="84"/>
+      <c r="EJ14" s="91"/>
       <c r="EK14" s="85"/>
       <c r="EL14" s="85"/>
       <c r="EM14" s="85"/>
@@ -4646,7 +4646,7 @@
       <c r="FM14" s="15"/>
       <c r="FN14" s="15"/>
       <c r="FO14" s="15"/>
-      <c r="FP14" s="101"/>
+      <c r="FP14" s="94"/>
     </row>
     <row r="15" spans="1:172" x14ac:dyDescent="0.2">
       <c r="A15" s="30" t="s">
@@ -4668,11 +4668,11 @@
       <c r="M15" s="15"/>
       <c r="N15" s="15"/>
       <c r="O15" s="15"/>
-      <c r="P15" s="94"/>
+      <c r="P15" s="84"/>
       <c r="Q15" s="85"/>
       <c r="R15" s="85"/>
       <c r="S15" s="86"/>
-      <c r="T15" s="84"/>
+      <c r="T15" s="91"/>
       <c r="U15" s="85"/>
       <c r="V15" s="85"/>
       <c r="W15" s="85"/>
@@ -4708,11 +4708,11 @@
       <c r="BA15" s="15"/>
       <c r="BB15" s="15"/>
       <c r="BC15" s="15"/>
-      <c r="BD15" s="94"/>
+      <c r="BD15" s="84"/>
       <c r="BE15" s="85"/>
       <c r="BF15" s="85"/>
       <c r="BG15" s="86"/>
-      <c r="BH15" s="84"/>
+      <c r="BH15" s="91"/>
       <c r="BI15" s="85"/>
       <c r="BJ15" s="85"/>
       <c r="BK15" s="85"/>
@@ -4720,7 +4720,7 @@
       <c r="BM15" s="85"/>
       <c r="BN15" s="85"/>
       <c r="BO15" s="86"/>
-      <c r="BP15" s="94"/>
+      <c r="BP15" s="84"/>
       <c r="BQ15" s="85"/>
       <c r="BR15" s="85"/>
       <c r="BS15" s="86"/>
@@ -4744,7 +4744,7 @@
       <c r="CK15" s="76"/>
       <c r="CL15" s="76"/>
       <c r="CM15" s="77"/>
-      <c r="CN15" s="84"/>
+      <c r="CN15" s="91"/>
       <c r="CO15" s="85"/>
       <c r="CP15" s="85"/>
       <c r="CQ15" s="85"/>
@@ -4788,11 +4788,11 @@
       <c r="EC15" s="15"/>
       <c r="ED15" s="15"/>
       <c r="EE15" s="15"/>
-      <c r="EF15" s="94"/>
+      <c r="EF15" s="84"/>
       <c r="EG15" s="85"/>
       <c r="EH15" s="85"/>
       <c r="EI15" s="86"/>
-      <c r="EJ15" s="84"/>
+      <c r="EJ15" s="91"/>
       <c r="EK15" s="85"/>
       <c r="EL15" s="85"/>
       <c r="EM15" s="85"/>
@@ -4824,7 +4824,7 @@
       <c r="FM15" s="15"/>
       <c r="FN15" s="15"/>
       <c r="FO15" s="15"/>
-      <c r="FP15" s="101"/>
+      <c r="FP15" s="94"/>
     </row>
     <row r="16" spans="1:172" x14ac:dyDescent="0.2">
       <c r="A16" s="12" t="s">
@@ -4848,11 +4848,11 @@
       <c r="M16" s="15"/>
       <c r="N16" s="15"/>
       <c r="O16" s="15"/>
-      <c r="P16" s="94"/>
+      <c r="P16" s="84"/>
       <c r="Q16" s="85"/>
       <c r="R16" s="85"/>
       <c r="S16" s="86"/>
-      <c r="T16" s="84"/>
+      <c r="T16" s="91"/>
       <c r="U16" s="85"/>
       <c r="V16" s="85"/>
       <c r="W16" s="85"/>
@@ -4888,11 +4888,11 @@
       <c r="BA16" s="15"/>
       <c r="BB16" s="15"/>
       <c r="BC16" s="15"/>
-      <c r="BD16" s="94"/>
+      <c r="BD16" s="84"/>
       <c r="BE16" s="85"/>
       <c r="BF16" s="85"/>
       <c r="BG16" s="86"/>
-      <c r="BH16" s="84"/>
+      <c r="BH16" s="91"/>
       <c r="BI16" s="85"/>
       <c r="BJ16" s="85"/>
       <c r="BK16" s="85"/>
@@ -4900,7 +4900,7 @@
       <c r="BM16" s="85"/>
       <c r="BN16" s="85"/>
       <c r="BO16" s="86"/>
-      <c r="BP16" s="94"/>
+      <c r="BP16" s="84"/>
       <c r="BQ16" s="85"/>
       <c r="BR16" s="85"/>
       <c r="BS16" s="86"/>
@@ -4924,7 +4924,7 @@
       <c r="CK16" s="76"/>
       <c r="CL16" s="76"/>
       <c r="CM16" s="77"/>
-      <c r="CN16" s="84"/>
+      <c r="CN16" s="91"/>
       <c r="CO16" s="85"/>
       <c r="CP16" s="85"/>
       <c r="CQ16" s="85"/>
@@ -4968,11 +4968,11 @@
       <c r="EC16" s="15"/>
       <c r="ED16" s="15"/>
       <c r="EE16" s="15"/>
-      <c r="EF16" s="94"/>
+      <c r="EF16" s="84"/>
       <c r="EG16" s="85"/>
       <c r="EH16" s="85"/>
       <c r="EI16" s="86"/>
-      <c r="EJ16" s="84"/>
+      <c r="EJ16" s="91"/>
       <c r="EK16" s="85"/>
       <c r="EL16" s="85"/>
       <c r="EM16" s="85"/>
@@ -5004,7 +5004,7 @@
       <c r="FM16" s="15"/>
       <c r="FN16" s="15"/>
       <c r="FO16" s="15"/>
-      <c r="FP16" s="101"/>
+      <c r="FP16" s="94"/>
     </row>
     <row r="17" spans="1:172 16352:16352" x14ac:dyDescent="0.2">
       <c r="A17" s="12" t="s">
@@ -5028,11 +5028,11 @@
         <v>46</v>
       </c>
       <c r="O17" s="46"/>
-      <c r="P17" s="94"/>
+      <c r="P17" s="84"/>
       <c r="Q17" s="85"/>
       <c r="R17" s="85"/>
       <c r="S17" s="86"/>
-      <c r="T17" s="84"/>
+      <c r="T17" s="91"/>
       <c r="U17" s="85"/>
       <c r="V17" s="85"/>
       <c r="W17" s="85"/>
@@ -5068,11 +5068,11 @@
       <c r="BA17" s="15"/>
       <c r="BB17" s="15"/>
       <c r="BC17" s="15"/>
-      <c r="BD17" s="94"/>
+      <c r="BD17" s="84"/>
       <c r="BE17" s="85"/>
       <c r="BF17" s="85"/>
       <c r="BG17" s="86"/>
-      <c r="BH17" s="84"/>
+      <c r="BH17" s="91"/>
       <c r="BI17" s="85"/>
       <c r="BJ17" s="85"/>
       <c r="BK17" s="85"/>
@@ -5080,7 +5080,7 @@
       <c r="BM17" s="85"/>
       <c r="BN17" s="85"/>
       <c r="BO17" s="86"/>
-      <c r="BP17" s="94"/>
+      <c r="BP17" s="84"/>
       <c r="BQ17" s="85"/>
       <c r="BR17" s="85"/>
       <c r="BS17" s="86"/>
@@ -5104,7 +5104,7 @@
       <c r="CK17" s="76"/>
       <c r="CL17" s="76"/>
       <c r="CM17" s="77"/>
-      <c r="CN17" s="84"/>
+      <c r="CN17" s="91"/>
       <c r="CO17" s="85"/>
       <c r="CP17" s="85"/>
       <c r="CQ17" s="85"/>
@@ -5148,11 +5148,11 @@
       <c r="EC17" s="15"/>
       <c r="ED17" s="15"/>
       <c r="EE17" s="15"/>
-      <c r="EF17" s="94"/>
+      <c r="EF17" s="84"/>
       <c r="EG17" s="85"/>
       <c r="EH17" s="85"/>
       <c r="EI17" s="86"/>
-      <c r="EJ17" s="84"/>
+      <c r="EJ17" s="91"/>
       <c r="EK17" s="85"/>
       <c r="EL17" s="85"/>
       <c r="EM17" s="85"/>
@@ -5184,7 +5184,7 @@
       <c r="FM17" s="15"/>
       <c r="FN17" s="15"/>
       <c r="FO17" s="15"/>
-      <c r="FP17" s="101"/>
+      <c r="FP17" s="94"/>
     </row>
     <row r="18" spans="1:172 16352:16352" x14ac:dyDescent="0.2">
       <c r="A18" s="41" t="s">
@@ -5208,11 +5208,11 @@
       <c r="O18" s="52" t="s">
         <v>46</v>
       </c>
-      <c r="P18" s="94"/>
+      <c r="P18" s="84"/>
       <c r="Q18" s="85"/>
       <c r="R18" s="85"/>
       <c r="S18" s="86"/>
-      <c r="T18" s="84"/>
+      <c r="T18" s="91"/>
       <c r="U18" s="85"/>
       <c r="V18" s="85"/>
       <c r="W18" s="85"/>
@@ -5248,11 +5248,11 @@
       <c r="BA18" s="15"/>
       <c r="BB18" s="15"/>
       <c r="BC18" s="15"/>
-      <c r="BD18" s="94"/>
+      <c r="BD18" s="84"/>
       <c r="BE18" s="85"/>
       <c r="BF18" s="85"/>
       <c r="BG18" s="86"/>
-      <c r="BH18" s="84"/>
+      <c r="BH18" s="91"/>
       <c r="BI18" s="85"/>
       <c r="BJ18" s="85"/>
       <c r="BK18" s="85"/>
@@ -5260,7 +5260,7 @@
       <c r="BM18" s="85"/>
       <c r="BN18" s="85"/>
       <c r="BO18" s="86"/>
-      <c r="BP18" s="94"/>
+      <c r="BP18" s="84"/>
       <c r="BQ18" s="85"/>
       <c r="BR18" s="85"/>
       <c r="BS18" s="86"/>
@@ -5284,7 +5284,7 @@
       <c r="CK18" s="76"/>
       <c r="CL18" s="76"/>
       <c r="CM18" s="77"/>
-      <c r="CN18" s="84"/>
+      <c r="CN18" s="91"/>
       <c r="CO18" s="85"/>
       <c r="CP18" s="85"/>
       <c r="CQ18" s="85"/>
@@ -5328,11 +5328,11 @@
       <c r="EC18" s="15"/>
       <c r="ED18" s="15"/>
       <c r="EE18" s="15"/>
-      <c r="EF18" s="94"/>
+      <c r="EF18" s="84"/>
       <c r="EG18" s="85"/>
       <c r="EH18" s="85"/>
       <c r="EI18" s="86"/>
-      <c r="EJ18" s="84"/>
+      <c r="EJ18" s="91"/>
       <c r="EK18" s="85"/>
       <c r="EL18" s="85"/>
       <c r="EM18" s="85"/>
@@ -5364,7 +5364,7 @@
       <c r="FM18" s="15"/>
       <c r="FN18" s="15"/>
       <c r="FO18" s="15"/>
-      <c r="FP18" s="101"/>
+      <c r="FP18" s="94"/>
     </row>
     <row r="19" spans="1:172 16352:16352" x14ac:dyDescent="0.2">
       <c r="A19" s="41" t="s">
@@ -5386,11 +5386,11 @@
       <c r="M19" s="15"/>
       <c r="N19" s="15"/>
       <c r="O19" s="46"/>
-      <c r="P19" s="94"/>
+      <c r="P19" s="84"/>
       <c r="Q19" s="85"/>
       <c r="R19" s="85"/>
       <c r="S19" s="86"/>
-      <c r="T19" s="84"/>
+      <c r="T19" s="91"/>
       <c r="U19" s="85"/>
       <c r="V19" s="85"/>
       <c r="W19" s="85"/>
@@ -5428,11 +5428,11 @@
       <c r="BA19" s="15"/>
       <c r="BB19" s="15"/>
       <c r="BC19" s="15"/>
-      <c r="BD19" s="94"/>
+      <c r="BD19" s="84"/>
       <c r="BE19" s="85"/>
       <c r="BF19" s="85"/>
       <c r="BG19" s="86"/>
-      <c r="BH19" s="84"/>
+      <c r="BH19" s="91"/>
       <c r="BI19" s="85"/>
       <c r="BJ19" s="85"/>
       <c r="BK19" s="85"/>
@@ -5440,7 +5440,7 @@
       <c r="BM19" s="85"/>
       <c r="BN19" s="85"/>
       <c r="BO19" s="86"/>
-      <c r="BP19" s="94"/>
+      <c r="BP19" s="84"/>
       <c r="BQ19" s="85"/>
       <c r="BR19" s="85"/>
       <c r="BS19" s="86"/>
@@ -5464,7 +5464,7 @@
       <c r="CK19" s="76"/>
       <c r="CL19" s="76"/>
       <c r="CM19" s="77"/>
-      <c r="CN19" s="84"/>
+      <c r="CN19" s="91"/>
       <c r="CO19" s="85"/>
       <c r="CP19" s="85"/>
       <c r="CQ19" s="85"/>
@@ -5508,11 +5508,11 @@
       <c r="EC19" s="15"/>
       <c r="ED19" s="15"/>
       <c r="EE19" s="15"/>
-      <c r="EF19" s="94"/>
+      <c r="EF19" s="84"/>
       <c r="EG19" s="85"/>
       <c r="EH19" s="85"/>
       <c r="EI19" s="86"/>
-      <c r="EJ19" s="84"/>
+      <c r="EJ19" s="91"/>
       <c r="EK19" s="85"/>
       <c r="EL19" s="85"/>
       <c r="EM19" s="85"/>
@@ -5544,7 +5544,7 @@
       <c r="FM19" s="15"/>
       <c r="FN19" s="15"/>
       <c r="FO19" s="15"/>
-      <c r="FP19" s="101"/>
+      <c r="FP19" s="94"/>
     </row>
     <row r="20" spans="1:172 16352:16352" x14ac:dyDescent="0.2">
       <c r="A20" s="53" t="s">
@@ -5566,11 +5566,11 @@
       <c r="M20" s="15"/>
       <c r="N20" s="15"/>
       <c r="O20" s="46"/>
-      <c r="P20" s="94"/>
+      <c r="P20" s="84"/>
       <c r="Q20" s="85"/>
       <c r="R20" s="85"/>
       <c r="S20" s="86"/>
-      <c r="T20" s="84"/>
+      <c r="T20" s="91"/>
       <c r="U20" s="85"/>
       <c r="V20" s="85"/>
       <c r="W20" s="85"/>
@@ -5608,11 +5608,11 @@
       <c r="BA20" s="15"/>
       <c r="BB20" s="15"/>
       <c r="BC20" s="15"/>
-      <c r="BD20" s="94"/>
+      <c r="BD20" s="84"/>
       <c r="BE20" s="85"/>
       <c r="BF20" s="85"/>
       <c r="BG20" s="86"/>
-      <c r="BH20" s="84"/>
+      <c r="BH20" s="91"/>
       <c r="BI20" s="85"/>
       <c r="BJ20" s="85"/>
       <c r="BK20" s="85"/>
@@ -5620,7 +5620,7 @@
       <c r="BM20" s="85"/>
       <c r="BN20" s="85"/>
       <c r="BO20" s="86"/>
-      <c r="BP20" s="94"/>
+      <c r="BP20" s="84"/>
       <c r="BQ20" s="85"/>
       <c r="BR20" s="85"/>
       <c r="BS20" s="86"/>
@@ -5644,7 +5644,7 @@
       <c r="CK20" s="76"/>
       <c r="CL20" s="76"/>
       <c r="CM20" s="77"/>
-      <c r="CN20" s="84"/>
+      <c r="CN20" s="91"/>
       <c r="CO20" s="85"/>
       <c r="CP20" s="85"/>
       <c r="CQ20" s="85"/>
@@ -5688,11 +5688,11 @@
       <c r="EC20" s="15"/>
       <c r="ED20" s="15"/>
       <c r="EE20" s="15"/>
-      <c r="EF20" s="94"/>
+      <c r="EF20" s="84"/>
       <c r="EG20" s="85"/>
       <c r="EH20" s="85"/>
       <c r="EI20" s="86"/>
-      <c r="EJ20" s="84"/>
+      <c r="EJ20" s="91"/>
       <c r="EK20" s="85"/>
       <c r="EL20" s="85"/>
       <c r="EM20" s="85"/>
@@ -5724,7 +5724,7 @@
       <c r="FM20" s="15"/>
       <c r="FN20" s="15"/>
       <c r="FO20" s="15"/>
-      <c r="FP20" s="101"/>
+      <c r="FP20" s="94"/>
     </row>
     <row r="21" spans="1:172 16352:16352" x14ac:dyDescent="0.2">
       <c r="A21" s="12" t="s">
@@ -5746,11 +5746,11 @@
       <c r="M21" s="15"/>
       <c r="N21" s="15"/>
       <c r="O21" s="15"/>
-      <c r="P21" s="94"/>
+      <c r="P21" s="84"/>
       <c r="Q21" s="85"/>
       <c r="R21" s="85"/>
       <c r="S21" s="86"/>
-      <c r="T21" s="84"/>
+      <c r="T21" s="91"/>
       <c r="U21" s="85"/>
       <c r="V21" s="85"/>
       <c r="W21" s="85"/>
@@ -5788,11 +5788,11 @@
       <c r="BA21" s="15"/>
       <c r="BB21" s="15"/>
       <c r="BC21" s="15"/>
-      <c r="BD21" s="94"/>
+      <c r="BD21" s="84"/>
       <c r="BE21" s="85"/>
       <c r="BF21" s="85"/>
       <c r="BG21" s="86"/>
-      <c r="BH21" s="84"/>
+      <c r="BH21" s="91"/>
       <c r="BI21" s="85"/>
       <c r="BJ21" s="85"/>
       <c r="BK21" s="85"/>
@@ -5800,7 +5800,7 @@
       <c r="BM21" s="85"/>
       <c r="BN21" s="85"/>
       <c r="BO21" s="86"/>
-      <c r="BP21" s="94"/>
+      <c r="BP21" s="84"/>
       <c r="BQ21" s="85"/>
       <c r="BR21" s="85"/>
       <c r="BS21" s="86"/>
@@ -5824,7 +5824,7 @@
       <c r="CK21" s="76"/>
       <c r="CL21" s="76"/>
       <c r="CM21" s="77"/>
-      <c r="CN21" s="84"/>
+      <c r="CN21" s="91"/>
       <c r="CO21" s="85"/>
       <c r="CP21" s="85"/>
       <c r="CQ21" s="85"/>
@@ -5868,11 +5868,11 @@
       <c r="EC21" s="15"/>
       <c r="ED21" s="15"/>
       <c r="EE21" s="15"/>
-      <c r="EF21" s="94"/>
+      <c r="EF21" s="84"/>
       <c r="EG21" s="85"/>
       <c r="EH21" s="85"/>
       <c r="EI21" s="86"/>
-      <c r="EJ21" s="84"/>
+      <c r="EJ21" s="91"/>
       <c r="EK21" s="85"/>
       <c r="EL21" s="85"/>
       <c r="EM21" s="85"/>
@@ -5904,7 +5904,7 @@
       <c r="FM21" s="15"/>
       <c r="FN21" s="15"/>
       <c r="FO21" s="15"/>
-      <c r="FP21" s="101"/>
+      <c r="FP21" s="94"/>
     </row>
     <row r="22" spans="1:172 16352:16352" x14ac:dyDescent="0.2">
       <c r="A22" s="12" t="s">
@@ -5926,11 +5926,11 @@
       <c r="M22" s="15"/>
       <c r="N22" s="15"/>
       <c r="O22" s="15"/>
-      <c r="P22" s="94"/>
+      <c r="P22" s="84"/>
       <c r="Q22" s="85"/>
       <c r="R22" s="85"/>
       <c r="S22" s="86"/>
-      <c r="T22" s="84"/>
+      <c r="T22" s="91"/>
       <c r="U22" s="85"/>
       <c r="V22" s="85"/>
       <c r="W22" s="85"/>
@@ -5970,11 +5970,11 @@
       <c r="BA22" s="15"/>
       <c r="BB22" s="15"/>
       <c r="BC22" s="15"/>
-      <c r="BD22" s="94"/>
+      <c r="BD22" s="84"/>
       <c r="BE22" s="85"/>
       <c r="BF22" s="85"/>
       <c r="BG22" s="86"/>
-      <c r="BH22" s="84"/>
+      <c r="BH22" s="91"/>
       <c r="BI22" s="85"/>
       <c r="BJ22" s="85"/>
       <c r="BK22" s="85"/>
@@ -5982,7 +5982,7 @@
       <c r="BM22" s="85"/>
       <c r="BN22" s="85"/>
       <c r="BO22" s="86"/>
-      <c r="BP22" s="94"/>
+      <c r="BP22" s="84"/>
       <c r="BQ22" s="85"/>
       <c r="BR22" s="85"/>
       <c r="BS22" s="86"/>
@@ -6006,7 +6006,7 @@
       <c r="CK22" s="76"/>
       <c r="CL22" s="76"/>
       <c r="CM22" s="77"/>
-      <c r="CN22" s="84"/>
+      <c r="CN22" s="91"/>
       <c r="CO22" s="85"/>
       <c r="CP22" s="85"/>
       <c r="CQ22" s="85"/>
@@ -6050,11 +6050,11 @@
       <c r="EC22" s="15"/>
       <c r="ED22" s="15"/>
       <c r="EE22" s="15"/>
-      <c r="EF22" s="94"/>
+      <c r="EF22" s="84"/>
       <c r="EG22" s="85"/>
       <c r="EH22" s="85"/>
       <c r="EI22" s="86"/>
-      <c r="EJ22" s="84"/>
+      <c r="EJ22" s="91"/>
       <c r="EK22" s="85"/>
       <c r="EL22" s="85"/>
       <c r="EM22" s="85"/>
@@ -6086,7 +6086,7 @@
       <c r="FM22" s="15"/>
       <c r="FN22" s="15"/>
       <c r="FO22" s="15"/>
-      <c r="FP22" s="101"/>
+      <c r="FP22" s="94"/>
     </row>
     <row r="23" spans="1:172 16352:16352" x14ac:dyDescent="0.2">
       <c r="A23" s="12" t="s">
@@ -6108,11 +6108,11 @@
       <c r="M23" s="15"/>
       <c r="N23" s="15"/>
       <c r="O23" s="15"/>
-      <c r="P23" s="94"/>
+      <c r="P23" s="84"/>
       <c r="Q23" s="85"/>
       <c r="R23" s="85"/>
       <c r="S23" s="86"/>
-      <c r="T23" s="84"/>
+      <c r="T23" s="91"/>
       <c r="U23" s="85"/>
       <c r="V23" s="85"/>
       <c r="W23" s="85"/>
@@ -6150,11 +6150,11 @@
       <c r="BA23" s="15"/>
       <c r="BB23" s="15"/>
       <c r="BC23" s="15"/>
-      <c r="BD23" s="94"/>
+      <c r="BD23" s="84"/>
       <c r="BE23" s="85"/>
       <c r="BF23" s="85"/>
       <c r="BG23" s="86"/>
-      <c r="BH23" s="84"/>
+      <c r="BH23" s="91"/>
       <c r="BI23" s="85"/>
       <c r="BJ23" s="85"/>
       <c r="BK23" s="85"/>
@@ -6162,7 +6162,7 @@
       <c r="BM23" s="85"/>
       <c r="BN23" s="85"/>
       <c r="BO23" s="86"/>
-      <c r="BP23" s="94"/>
+      <c r="BP23" s="84"/>
       <c r="BQ23" s="85"/>
       <c r="BR23" s="85"/>
       <c r="BS23" s="86"/>
@@ -6186,7 +6186,7 @@
       <c r="CK23" s="76"/>
       <c r="CL23" s="76"/>
       <c r="CM23" s="77"/>
-      <c r="CN23" s="84"/>
+      <c r="CN23" s="91"/>
       <c r="CO23" s="85"/>
       <c r="CP23" s="85"/>
       <c r="CQ23" s="85"/>
@@ -6230,11 +6230,11 @@
       <c r="EC23" s="15"/>
       <c r="ED23" s="15"/>
       <c r="EE23" s="15"/>
-      <c r="EF23" s="94"/>
+      <c r="EF23" s="84"/>
       <c r="EG23" s="85"/>
       <c r="EH23" s="85"/>
       <c r="EI23" s="86"/>
-      <c r="EJ23" s="84"/>
+      <c r="EJ23" s="91"/>
       <c r="EK23" s="85"/>
       <c r="EL23" s="85"/>
       <c r="EM23" s="85"/>
@@ -6266,7 +6266,7 @@
       <c r="FM23" s="15"/>
       <c r="FN23" s="15"/>
       <c r="FO23" s="15"/>
-      <c r="FP23" s="101"/>
+      <c r="FP23" s="94"/>
     </row>
     <row r="24" spans="1:172 16352:16352" x14ac:dyDescent="0.2">
       <c r="A24" s="12" t="s">
@@ -6288,11 +6288,11 @@
       <c r="M24" s="15"/>
       <c r="N24" s="15"/>
       <c r="O24" s="15"/>
-      <c r="P24" s="94"/>
+      <c r="P24" s="84"/>
       <c r="Q24" s="85"/>
       <c r="R24" s="85"/>
       <c r="S24" s="86"/>
-      <c r="T24" s="84"/>
+      <c r="T24" s="91"/>
       <c r="U24" s="85"/>
       <c r="V24" s="85"/>
       <c r="W24" s="85"/>
@@ -6329,11 +6329,11 @@
       <c r="BA24" s="15"/>
       <c r="BB24" s="15"/>
       <c r="BC24" s="15"/>
-      <c r="BD24" s="94"/>
+      <c r="BD24" s="84"/>
       <c r="BE24" s="85"/>
       <c r="BF24" s="85"/>
       <c r="BG24" s="86"/>
-      <c r="BH24" s="84"/>
+      <c r="BH24" s="91"/>
       <c r="BI24" s="85"/>
       <c r="BJ24" s="85"/>
       <c r="BK24" s="85"/>
@@ -6341,7 +6341,7 @@
       <c r="BM24" s="85"/>
       <c r="BN24" s="85"/>
       <c r="BO24" s="86"/>
-      <c r="BP24" s="94"/>
+      <c r="BP24" s="84"/>
       <c r="BQ24" s="85"/>
       <c r="BR24" s="85"/>
       <c r="BS24" s="86"/>
@@ -6365,7 +6365,7 @@
       <c r="CK24" s="76"/>
       <c r="CL24" s="76"/>
       <c r="CM24" s="77"/>
-      <c r="CN24" s="84"/>
+      <c r="CN24" s="91"/>
       <c r="CO24" s="85"/>
       <c r="CP24" s="85"/>
       <c r="CQ24" s="85"/>
@@ -6409,11 +6409,11 @@
       <c r="EC24" s="15"/>
       <c r="ED24" s="15"/>
       <c r="EE24" s="15"/>
-      <c r="EF24" s="94"/>
+      <c r="EF24" s="84"/>
       <c r="EG24" s="85"/>
       <c r="EH24" s="85"/>
       <c r="EI24" s="86"/>
-      <c r="EJ24" s="84"/>
+      <c r="EJ24" s="91"/>
       <c r="EK24" s="85"/>
       <c r="EL24" s="85"/>
       <c r="EM24" s="85"/>
@@ -6445,7 +6445,7 @@
       <c r="FM24" s="15"/>
       <c r="FN24" s="15"/>
       <c r="FO24" s="15"/>
-      <c r="FP24" s="101"/>
+      <c r="FP24" s="94"/>
     </row>
     <row r="25" spans="1:172 16352:16352" x14ac:dyDescent="0.2">
       <c r="B25" s="23"/>
@@ -6462,11 +6462,11 @@
       <c r="M25" s="15"/>
       <c r="N25" s="15"/>
       <c r="O25" s="15"/>
-      <c r="P25" s="94"/>
+      <c r="P25" s="84"/>
       <c r="Q25" s="85"/>
       <c r="R25" s="85"/>
       <c r="S25" s="86"/>
-      <c r="T25" s="84"/>
+      <c r="T25" s="91"/>
       <c r="U25" s="85"/>
       <c r="V25" s="85"/>
       <c r="W25" s="85"/>
@@ -6502,11 +6502,11 @@
       <c r="BA25" s="15"/>
       <c r="BB25" s="15"/>
       <c r="BC25" s="15"/>
-      <c r="BD25" s="94"/>
+      <c r="BD25" s="84"/>
       <c r="BE25" s="85"/>
       <c r="BF25" s="85"/>
       <c r="BG25" s="86"/>
-      <c r="BH25" s="84"/>
+      <c r="BH25" s="91"/>
       <c r="BI25" s="85"/>
       <c r="BJ25" s="85"/>
       <c r="BK25" s="85"/>
@@ -6514,7 +6514,7 @@
       <c r="BM25" s="85"/>
       <c r="BN25" s="85"/>
       <c r="BO25" s="86"/>
-      <c r="BP25" s="94"/>
+      <c r="BP25" s="84"/>
       <c r="BQ25" s="85"/>
       <c r="BR25" s="85"/>
       <c r="BS25" s="86"/>
@@ -6538,7 +6538,7 @@
       <c r="CK25" s="76"/>
       <c r="CL25" s="76"/>
       <c r="CM25" s="77"/>
-      <c r="CN25" s="84"/>
+      <c r="CN25" s="91"/>
       <c r="CO25" s="85"/>
       <c r="CP25" s="85"/>
       <c r="CQ25" s="85"/>
@@ -6582,11 +6582,11 @@
       <c r="EC25" s="15"/>
       <c r="ED25" s="15"/>
       <c r="EE25" s="15"/>
-      <c r="EF25" s="94"/>
+      <c r="EF25" s="84"/>
       <c r="EG25" s="85"/>
       <c r="EH25" s="85"/>
       <c r="EI25" s="86"/>
-      <c r="EJ25" s="84"/>
+      <c r="EJ25" s="91"/>
       <c r="EK25" s="85"/>
       <c r="EL25" s="85"/>
       <c r="EM25" s="85"/>
@@ -6618,7 +6618,7 @@
       <c r="FM25" s="15"/>
       <c r="FN25" s="15"/>
       <c r="FO25" s="15"/>
-      <c r="FP25" s="101"/>
+      <c r="FP25" s="94"/>
     </row>
     <row r="26" spans="1:172 16352:16352" x14ac:dyDescent="0.2">
       <c r="A26" s="31" t="s">
@@ -6640,11 +6640,11 @@
       <c r="M26" s="15"/>
       <c r="N26" s="15"/>
       <c r="O26" s="15"/>
-      <c r="P26" s="94"/>
+      <c r="P26" s="84"/>
       <c r="Q26" s="85"/>
       <c r="R26" s="85"/>
       <c r="S26" s="86"/>
-      <c r="T26" s="84"/>
+      <c r="T26" s="91"/>
       <c r="U26" s="85"/>
       <c r="V26" s="85"/>
       <c r="W26" s="85"/>
@@ -6680,11 +6680,11 @@
       <c r="BA26" s="15"/>
       <c r="BB26" s="15"/>
       <c r="BC26" s="15"/>
-      <c r="BD26" s="94"/>
+      <c r="BD26" s="84"/>
       <c r="BE26" s="85"/>
       <c r="BF26" s="85"/>
       <c r="BG26" s="86"/>
-      <c r="BH26" s="84"/>
+      <c r="BH26" s="91"/>
       <c r="BI26" s="85"/>
       <c r="BJ26" s="85"/>
       <c r="BK26" s="85"/>
@@ -6692,7 +6692,7 @@
       <c r="BM26" s="85"/>
       <c r="BN26" s="85"/>
       <c r="BO26" s="86"/>
-      <c r="BP26" s="94"/>
+      <c r="BP26" s="84"/>
       <c r="BQ26" s="85"/>
       <c r="BR26" s="85"/>
       <c r="BS26" s="86"/>
@@ -6716,7 +6716,7 @@
       <c r="CK26" s="76"/>
       <c r="CL26" s="76"/>
       <c r="CM26" s="77"/>
-      <c r="CN26" s="84"/>
+      <c r="CN26" s="91"/>
       <c r="CO26" s="85"/>
       <c r="CP26" s="85"/>
       <c r="CQ26" s="85"/>
@@ -6760,11 +6760,11 @@
       <c r="EC26" s="15"/>
       <c r="ED26" s="15"/>
       <c r="EE26" s="15"/>
-      <c r="EF26" s="94"/>
+      <c r="EF26" s="84"/>
       <c r="EG26" s="85"/>
       <c r="EH26" s="85"/>
       <c r="EI26" s="86"/>
-      <c r="EJ26" s="84"/>
+      <c r="EJ26" s="91"/>
       <c r="EK26" s="85"/>
       <c r="EL26" s="85"/>
       <c r="EM26" s="85"/>
@@ -6796,7 +6796,7 @@
       <c r="FM26" s="15"/>
       <c r="FN26" s="15"/>
       <c r="FO26" s="15"/>
-      <c r="FP26" s="101"/>
+      <c r="FP26" s="94"/>
     </row>
     <row r="27" spans="1:172 16352:16352" x14ac:dyDescent="0.2">
       <c r="A27" s="55" t="s">
@@ -6818,11 +6818,11 @@
       <c r="M27" s="15"/>
       <c r="N27" s="15"/>
       <c r="O27" s="15"/>
-      <c r="P27" s="94"/>
+      <c r="P27" s="84"/>
       <c r="Q27" s="85"/>
       <c r="R27" s="85"/>
       <c r="S27" s="86"/>
-      <c r="T27" s="84"/>
+      <c r="T27" s="91"/>
       <c r="U27" s="85"/>
       <c r="V27" s="85"/>
       <c r="W27" s="85"/>
@@ -6860,11 +6860,11 @@
       <c r="BA27" s="15"/>
       <c r="BB27" s="15"/>
       <c r="BC27" s="15"/>
-      <c r="BD27" s="94"/>
+      <c r="BD27" s="84"/>
       <c r="BE27" s="85"/>
       <c r="BF27" s="85"/>
       <c r="BG27" s="86"/>
-      <c r="BH27" s="84"/>
+      <c r="BH27" s="91"/>
       <c r="BI27" s="85"/>
       <c r="BJ27" s="85"/>
       <c r="BK27" s="85"/>
@@ -6872,7 +6872,7 @@
       <c r="BM27" s="85"/>
       <c r="BN27" s="85"/>
       <c r="BO27" s="86"/>
-      <c r="BP27" s="94"/>
+      <c r="BP27" s="84"/>
       <c r="BQ27" s="85"/>
       <c r="BR27" s="85"/>
       <c r="BS27" s="86"/>
@@ -6896,7 +6896,7 @@
       <c r="CK27" s="76"/>
       <c r="CL27" s="76"/>
       <c r="CM27" s="77"/>
-      <c r="CN27" s="84"/>
+      <c r="CN27" s="91"/>
       <c r="CO27" s="85"/>
       <c r="CP27" s="85"/>
       <c r="CQ27" s="85"/>
@@ -6940,11 +6940,11 @@
       <c r="EC27" s="15"/>
       <c r="ED27" s="15"/>
       <c r="EE27" s="15"/>
-      <c r="EF27" s="94"/>
+      <c r="EF27" s="84"/>
       <c r="EG27" s="85"/>
       <c r="EH27" s="85"/>
       <c r="EI27" s="86"/>
-      <c r="EJ27" s="84"/>
+      <c r="EJ27" s="91"/>
       <c r="EK27" s="85"/>
       <c r="EL27" s="85"/>
       <c r="EM27" s="85"/>
@@ -6976,7 +6976,7 @@
       <c r="FM27" s="15"/>
       <c r="FN27" s="15"/>
       <c r="FO27" s="15"/>
-      <c r="FP27" s="101"/>
+      <c r="FP27" s="94"/>
     </row>
     <row r="28" spans="1:172 16352:16352" x14ac:dyDescent="0.2">
       <c r="A28" s="54" t="s">
@@ -6998,11 +6998,11 @@
       <c r="M28" s="15"/>
       <c r="N28" s="15"/>
       <c r="O28" s="15"/>
-      <c r="P28" s="94"/>
+      <c r="P28" s="84"/>
       <c r="Q28" s="85"/>
       <c r="R28" s="85"/>
       <c r="S28" s="86"/>
-      <c r="T28" s="84"/>
+      <c r="T28" s="91"/>
       <c r="U28" s="85"/>
       <c r="V28" s="85"/>
       <c r="W28" s="85"/>
@@ -7040,11 +7040,11 @@
       <c r="BA28" s="15"/>
       <c r="BB28" s="15"/>
       <c r="BC28" s="15"/>
-      <c r="BD28" s="94"/>
+      <c r="BD28" s="84"/>
       <c r="BE28" s="85"/>
       <c r="BF28" s="85"/>
       <c r="BG28" s="86"/>
-      <c r="BH28" s="84"/>
+      <c r="BH28" s="91"/>
       <c r="BI28" s="85"/>
       <c r="BJ28" s="85"/>
       <c r="BK28" s="85"/>
@@ -7052,7 +7052,7 @@
       <c r="BM28" s="85"/>
       <c r="BN28" s="85"/>
       <c r="BO28" s="86"/>
-      <c r="BP28" s="94"/>
+      <c r="BP28" s="84"/>
       <c r="BQ28" s="85"/>
       <c r="BR28" s="85"/>
       <c r="BS28" s="86"/>
@@ -7076,7 +7076,7 @@
       <c r="CK28" s="76"/>
       <c r="CL28" s="76"/>
       <c r="CM28" s="77"/>
-      <c r="CN28" s="84"/>
+      <c r="CN28" s="91"/>
       <c r="CO28" s="85"/>
       <c r="CP28" s="85"/>
       <c r="CQ28" s="85"/>
@@ -7120,11 +7120,11 @@
       <c r="EC28" s="15"/>
       <c r="ED28" s="15"/>
       <c r="EE28" s="15"/>
-      <c r="EF28" s="94"/>
+      <c r="EF28" s="84"/>
       <c r="EG28" s="85"/>
       <c r="EH28" s="85"/>
       <c r="EI28" s="86"/>
-      <c r="EJ28" s="84"/>
+      <c r="EJ28" s="91"/>
       <c r="EK28" s="85"/>
       <c r="EL28" s="85"/>
       <c r="EM28" s="85"/>
@@ -7156,7 +7156,7 @@
       <c r="FM28" s="15"/>
       <c r="FN28" s="15"/>
       <c r="FO28" s="15"/>
-      <c r="FP28" s="101"/>
+      <c r="FP28" s="94"/>
       <c r="XDX28" s="40"/>
     </row>
     <row r="29" spans="1:172 16352:16352" x14ac:dyDescent="0.2">
@@ -7179,11 +7179,11 @@
       <c r="M29" s="15"/>
       <c r="N29" s="15"/>
       <c r="O29" s="15"/>
-      <c r="P29" s="94"/>
+      <c r="P29" s="84"/>
       <c r="Q29" s="85"/>
       <c r="R29" s="85"/>
       <c r="S29" s="86"/>
-      <c r="T29" s="84"/>
+      <c r="T29" s="91"/>
       <c r="U29" s="85"/>
       <c r="V29" s="85"/>
       <c r="W29" s="85"/>
@@ -7223,11 +7223,11 @@
       <c r="BA29" s="15"/>
       <c r="BB29" s="15"/>
       <c r="BC29" s="15"/>
-      <c r="BD29" s="94"/>
+      <c r="BD29" s="84"/>
       <c r="BE29" s="85"/>
       <c r="BF29" s="85"/>
       <c r="BG29" s="86"/>
-      <c r="BH29" s="84"/>
+      <c r="BH29" s="91"/>
       <c r="BI29" s="85"/>
       <c r="BJ29" s="85"/>
       <c r="BK29" s="85"/>
@@ -7235,7 +7235,7 @@
       <c r="BM29" s="85"/>
       <c r="BN29" s="85"/>
       <c r="BO29" s="86"/>
-      <c r="BP29" s="94"/>
+      <c r="BP29" s="84"/>
       <c r="BQ29" s="85"/>
       <c r="BR29" s="85"/>
       <c r="BS29" s="86"/>
@@ -7259,7 +7259,7 @@
       <c r="CK29" s="76"/>
       <c r="CL29" s="76"/>
       <c r="CM29" s="77"/>
-      <c r="CN29" s="84"/>
+      <c r="CN29" s="91"/>
       <c r="CO29" s="85"/>
       <c r="CP29" s="85"/>
       <c r="CQ29" s="85"/>
@@ -7307,11 +7307,11 @@
       <c r="EC29" s="15"/>
       <c r="ED29" s="15"/>
       <c r="EE29" s="15"/>
-      <c r="EF29" s="94"/>
+      <c r="EF29" s="84"/>
       <c r="EG29" s="85"/>
       <c r="EH29" s="85"/>
       <c r="EI29" s="86"/>
-      <c r="EJ29" s="84"/>
+      <c r="EJ29" s="91"/>
       <c r="EK29" s="85"/>
       <c r="EL29" s="85"/>
       <c r="EM29" s="85"/>
@@ -7343,7 +7343,7 @@
       <c r="FM29" s="15"/>
       <c r="FN29" s="15"/>
       <c r="FO29" s="15"/>
-      <c r="FP29" s="101"/>
+      <c r="FP29" s="94"/>
     </row>
     <row r="30" spans="1:172 16352:16352" x14ac:dyDescent="0.2">
       <c r="A30" s="12" t="s">
@@ -7365,11 +7365,11 @@
       <c r="M30" s="15"/>
       <c r="N30" s="15"/>
       <c r="O30" s="15"/>
-      <c r="P30" s="94"/>
+      <c r="P30" s="84"/>
       <c r="Q30" s="85"/>
       <c r="R30" s="85"/>
       <c r="S30" s="86"/>
-      <c r="T30" s="84"/>
+      <c r="T30" s="91"/>
       <c r="U30" s="85"/>
       <c r="V30" s="85"/>
       <c r="W30" s="85"/>
@@ -7407,11 +7407,11 @@
       <c r="BA30" s="40"/>
       <c r="BB30" s="15"/>
       <c r="BC30" s="15"/>
-      <c r="BD30" s="94"/>
+      <c r="BD30" s="84"/>
       <c r="BE30" s="85"/>
       <c r="BF30" s="85"/>
       <c r="BG30" s="86"/>
-      <c r="BH30" s="84"/>
+      <c r="BH30" s="91"/>
       <c r="BI30" s="85"/>
       <c r="BJ30" s="85"/>
       <c r="BK30" s="85"/>
@@ -7419,7 +7419,7 @@
       <c r="BM30" s="85"/>
       <c r="BN30" s="85"/>
       <c r="BO30" s="86"/>
-      <c r="BP30" s="94"/>
+      <c r="BP30" s="84"/>
       <c r="BQ30" s="85"/>
       <c r="BR30" s="85"/>
       <c r="BS30" s="86"/>
@@ -7443,7 +7443,7 @@
       <c r="CK30" s="76"/>
       <c r="CL30" s="76"/>
       <c r="CM30" s="77"/>
-      <c r="CN30" s="84"/>
+      <c r="CN30" s="91"/>
       <c r="CO30" s="85"/>
       <c r="CP30" s="85"/>
       <c r="CQ30" s="85"/>
@@ -7487,11 +7487,11 @@
       <c r="EC30" s="15"/>
       <c r="ED30" s="15"/>
       <c r="EE30" s="15"/>
-      <c r="EF30" s="94"/>
+      <c r="EF30" s="84"/>
       <c r="EG30" s="85"/>
       <c r="EH30" s="85"/>
       <c r="EI30" s="86"/>
-      <c r="EJ30" s="84"/>
+      <c r="EJ30" s="91"/>
       <c r="EK30" s="85"/>
       <c r="EL30" s="85"/>
       <c r="EM30" s="85"/>
@@ -7523,7 +7523,7 @@
       <c r="FM30" s="15"/>
       <c r="FN30" s="15"/>
       <c r="FO30" s="15"/>
-      <c r="FP30" s="101"/>
+      <c r="FP30" s="94"/>
     </row>
     <row r="31" spans="1:172 16352:16352" x14ac:dyDescent="0.2">
       <c r="A31" s="12" t="s">
@@ -7545,11 +7545,11 @@
       <c r="M31" s="15"/>
       <c r="N31" s="15"/>
       <c r="O31" s="15"/>
-      <c r="P31" s="94"/>
+      <c r="P31" s="84"/>
       <c r="Q31" s="85"/>
       <c r="R31" s="85"/>
       <c r="S31" s="86"/>
-      <c r="T31" s="84"/>
+      <c r="T31" s="91"/>
       <c r="U31" s="85"/>
       <c r="V31" s="85"/>
       <c r="W31" s="85"/>
@@ -7587,11 +7587,11 @@
       <c r="BA31" s="15"/>
       <c r="BB31" s="40"/>
       <c r="BC31" s="40"/>
-      <c r="BD31" s="94"/>
+      <c r="BD31" s="84"/>
       <c r="BE31" s="85"/>
       <c r="BF31" s="85"/>
       <c r="BG31" s="86"/>
-      <c r="BH31" s="84"/>
+      <c r="BH31" s="91"/>
       <c r="BI31" s="85"/>
       <c r="BJ31" s="85"/>
       <c r="BK31" s="85"/>
@@ -7599,7 +7599,7 @@
       <c r="BM31" s="85"/>
       <c r="BN31" s="85"/>
       <c r="BO31" s="86"/>
-      <c r="BP31" s="94"/>
+      <c r="BP31" s="84"/>
       <c r="BQ31" s="85"/>
       <c r="BR31" s="85"/>
       <c r="BS31" s="86"/>
@@ -7623,7 +7623,7 @@
       <c r="CK31" s="76"/>
       <c r="CL31" s="76"/>
       <c r="CM31" s="77"/>
-      <c r="CN31" s="84"/>
+      <c r="CN31" s="91"/>
       <c r="CO31" s="85"/>
       <c r="CP31" s="85"/>
       <c r="CQ31" s="85"/>
@@ -7667,11 +7667,11 @@
       <c r="EC31" s="15"/>
       <c r="ED31" s="15"/>
       <c r="EE31" s="15"/>
-      <c r="EF31" s="94"/>
+      <c r="EF31" s="84"/>
       <c r="EG31" s="85"/>
       <c r="EH31" s="85"/>
       <c r="EI31" s="86"/>
-      <c r="EJ31" s="84"/>
+      <c r="EJ31" s="91"/>
       <c r="EK31" s="85"/>
       <c r="EL31" s="85"/>
       <c r="EM31" s="85"/>
@@ -7703,7 +7703,7 @@
       <c r="FM31" s="15"/>
       <c r="FN31" s="15"/>
       <c r="FO31" s="15"/>
-      <c r="FP31" s="101"/>
+      <c r="FP31" s="94"/>
     </row>
     <row r="32" spans="1:172 16352:16352" x14ac:dyDescent="0.2">
       <c r="A32" s="41" t="s">
@@ -7725,11 +7725,11 @@
       <c r="M32" s="15"/>
       <c r="N32" s="15"/>
       <c r="O32" s="15"/>
-      <c r="P32" s="94"/>
+      <c r="P32" s="84"/>
       <c r="Q32" s="85"/>
       <c r="R32" s="85"/>
       <c r="S32" s="86"/>
-      <c r="T32" s="84"/>
+      <c r="T32" s="91"/>
       <c r="U32" s="85"/>
       <c r="V32" s="85"/>
       <c r="W32" s="85"/>
@@ -7767,11 +7767,11 @@
       <c r="BA32" s="15"/>
       <c r="BB32" s="15"/>
       <c r="BC32" s="15"/>
-      <c r="BD32" s="94"/>
+      <c r="BD32" s="84"/>
       <c r="BE32" s="85"/>
       <c r="BF32" s="85"/>
       <c r="BG32" s="86"/>
-      <c r="BH32" s="84"/>
+      <c r="BH32" s="91"/>
       <c r="BI32" s="85"/>
       <c r="BJ32" s="85"/>
       <c r="BK32" s="85"/>
@@ -7779,7 +7779,7 @@
       <c r="BM32" s="85"/>
       <c r="BN32" s="85"/>
       <c r="BO32" s="86"/>
-      <c r="BP32" s="94"/>
+      <c r="BP32" s="84"/>
       <c r="BQ32" s="85"/>
       <c r="BR32" s="85"/>
       <c r="BS32" s="86"/>
@@ -7803,7 +7803,7 @@
       <c r="CK32" s="76"/>
       <c r="CL32" s="76"/>
       <c r="CM32" s="77"/>
-      <c r="CN32" s="84"/>
+      <c r="CN32" s="91"/>
       <c r="CO32" s="85"/>
       <c r="CP32" s="85"/>
       <c r="CQ32" s="85"/>
@@ -7847,11 +7847,11 @@
       <c r="EC32" s="15"/>
       <c r="ED32" s="15"/>
       <c r="EE32" s="15"/>
-      <c r="EF32" s="94"/>
+      <c r="EF32" s="84"/>
       <c r="EG32" s="85"/>
       <c r="EH32" s="85"/>
       <c r="EI32" s="86"/>
-      <c r="EJ32" s="84"/>
+      <c r="EJ32" s="91"/>
       <c r="EK32" s="85"/>
       <c r="EL32" s="85"/>
       <c r="EM32" s="85"/>
@@ -7883,7 +7883,7 @@
       <c r="FM32" s="15"/>
       <c r="FN32" s="15"/>
       <c r="FO32" s="15"/>
-      <c r="FP32" s="101"/>
+      <c r="FP32" s="94"/>
     </row>
     <row r="33" spans="1:172" x14ac:dyDescent="0.2">
       <c r="A33" s="41" t="s">
@@ -7905,11 +7905,11 @@
       <c r="M33" s="15"/>
       <c r="N33" s="15"/>
       <c r="O33" s="15"/>
-      <c r="P33" s="94"/>
+      <c r="P33" s="84"/>
       <c r="Q33" s="85"/>
       <c r="R33" s="85"/>
       <c r="S33" s="86"/>
-      <c r="T33" s="84"/>
+      <c r="T33" s="91"/>
       <c r="U33" s="85"/>
       <c r="V33" s="85"/>
       <c r="W33" s="85"/>
@@ -7949,11 +7949,11 @@
       <c r="BA33" s="15"/>
       <c r="BB33" s="15"/>
       <c r="BC33" s="15"/>
-      <c r="BD33" s="94"/>
+      <c r="BD33" s="84"/>
       <c r="BE33" s="85"/>
       <c r="BF33" s="85"/>
       <c r="BG33" s="86"/>
-      <c r="BH33" s="84"/>
+      <c r="BH33" s="91"/>
       <c r="BI33" s="85"/>
       <c r="BJ33" s="85"/>
       <c r="BK33" s="85"/>
@@ -7961,7 +7961,7 @@
       <c r="BM33" s="85"/>
       <c r="BN33" s="85"/>
       <c r="BO33" s="86"/>
-      <c r="BP33" s="94"/>
+      <c r="BP33" s="84"/>
       <c r="BQ33" s="85"/>
       <c r="BR33" s="85"/>
       <c r="BS33" s="86"/>
@@ -7985,7 +7985,7 @@
       <c r="CK33" s="76"/>
       <c r="CL33" s="76"/>
       <c r="CM33" s="77"/>
-      <c r="CN33" s="84"/>
+      <c r="CN33" s="91"/>
       <c r="CO33" s="85"/>
       <c r="CP33" s="85"/>
       <c r="CQ33" s="85"/>
@@ -8029,11 +8029,11 @@
       <c r="EC33" s="15"/>
       <c r="ED33" s="15"/>
       <c r="EE33" s="15"/>
-      <c r="EF33" s="94"/>
+      <c r="EF33" s="84"/>
       <c r="EG33" s="85"/>
       <c r="EH33" s="85"/>
       <c r="EI33" s="86"/>
-      <c r="EJ33" s="84"/>
+      <c r="EJ33" s="91"/>
       <c r="EK33" s="85"/>
       <c r="EL33" s="85"/>
       <c r="EM33" s="85"/>
@@ -8065,7 +8065,7 @@
       <c r="FM33" s="15"/>
       <c r="FN33" s="15"/>
       <c r="FO33" s="15"/>
-      <c r="FP33" s="101"/>
+      <c r="FP33" s="94"/>
     </row>
     <row r="34" spans="1:172" x14ac:dyDescent="0.2">
       <c r="A34" s="41" t="s">
@@ -8087,11 +8087,11 @@
       <c r="M34" s="15"/>
       <c r="N34" s="15"/>
       <c r="O34" s="15"/>
-      <c r="P34" s="94"/>
+      <c r="P34" s="84"/>
       <c r="Q34" s="85"/>
       <c r="R34" s="85"/>
       <c r="S34" s="86"/>
-      <c r="T34" s="84"/>
+      <c r="T34" s="91"/>
       <c r="U34" s="85"/>
       <c r="V34" s="85"/>
       <c r="W34" s="85"/>
@@ -8131,11 +8131,11 @@
       <c r="BA34" s="15"/>
       <c r="BB34" s="15"/>
       <c r="BC34" s="15"/>
-      <c r="BD34" s="94"/>
+      <c r="BD34" s="84"/>
       <c r="BE34" s="85"/>
       <c r="BF34" s="85"/>
       <c r="BG34" s="86"/>
-      <c r="BH34" s="84"/>
+      <c r="BH34" s="91"/>
       <c r="BI34" s="85"/>
       <c r="BJ34" s="85"/>
       <c r="BK34" s="85"/>
@@ -8143,7 +8143,7 @@
       <c r="BM34" s="85"/>
       <c r="BN34" s="85"/>
       <c r="BO34" s="86"/>
-      <c r="BP34" s="94"/>
+      <c r="BP34" s="84"/>
       <c r="BQ34" s="85"/>
       <c r="BR34" s="85"/>
       <c r="BS34" s="86"/>
@@ -8167,7 +8167,7 @@
       <c r="CK34" s="76"/>
       <c r="CL34" s="76"/>
       <c r="CM34" s="77"/>
-      <c r="CN34" s="84"/>
+      <c r="CN34" s="91"/>
       <c r="CO34" s="85"/>
       <c r="CP34" s="85"/>
       <c r="CQ34" s="85"/>
@@ -8211,11 +8211,11 @@
       <c r="EC34" s="15"/>
       <c r="ED34" s="15"/>
       <c r="EE34" s="15"/>
-      <c r="EF34" s="94"/>
+      <c r="EF34" s="84"/>
       <c r="EG34" s="85"/>
       <c r="EH34" s="85"/>
       <c r="EI34" s="86"/>
-      <c r="EJ34" s="84"/>
+      <c r="EJ34" s="91"/>
       <c r="EK34" s="85"/>
       <c r="EL34" s="85"/>
       <c r="EM34" s="85"/>
@@ -8247,7 +8247,7 @@
       <c r="FM34" s="15"/>
       <c r="FN34" s="15"/>
       <c r="FO34" s="15"/>
-      <c r="FP34" s="101"/>
+      <c r="FP34" s="94"/>
     </row>
     <row r="35" spans="1:172" x14ac:dyDescent="0.2">
       <c r="A35" s="41" t="s">
@@ -8269,11 +8269,11 @@
       <c r="M35" s="36"/>
       <c r="N35" s="36"/>
       <c r="O35" s="36"/>
-      <c r="P35" s="94"/>
+      <c r="P35" s="84"/>
       <c r="Q35" s="85"/>
       <c r="R35" s="85"/>
       <c r="S35" s="86"/>
-      <c r="T35" s="84"/>
+      <c r="T35" s="91"/>
       <c r="U35" s="85"/>
       <c r="V35" s="85"/>
       <c r="W35" s="85"/>
@@ -8319,11 +8319,11 @@
         <v>46</v>
       </c>
       <c r="BC35" s="36"/>
-      <c r="BD35" s="94"/>
+      <c r="BD35" s="84"/>
       <c r="BE35" s="85"/>
       <c r="BF35" s="85"/>
       <c r="BG35" s="86"/>
-      <c r="BH35" s="84"/>
+      <c r="BH35" s="91"/>
       <c r="BI35" s="85"/>
       <c r="BJ35" s="85"/>
       <c r="BK35" s="85"/>
@@ -8331,7 +8331,7 @@
       <c r="BM35" s="85"/>
       <c r="BN35" s="85"/>
       <c r="BO35" s="86"/>
-      <c r="BP35" s="94"/>
+      <c r="BP35" s="84"/>
       <c r="BQ35" s="85"/>
       <c r="BR35" s="85"/>
       <c r="BS35" s="86"/>
@@ -8363,7 +8363,7 @@
       <c r="CK35" s="76"/>
       <c r="CL35" s="76"/>
       <c r="CM35" s="77"/>
-      <c r="CN35" s="84"/>
+      <c r="CN35" s="91"/>
       <c r="CO35" s="85"/>
       <c r="CP35" s="85"/>
       <c r="CQ35" s="85"/>
@@ -8407,11 +8407,11 @@
       <c r="EC35" s="36"/>
       <c r="ED35" s="36"/>
       <c r="EE35" s="36"/>
-      <c r="EF35" s="94"/>
+      <c r="EF35" s="84"/>
       <c r="EG35" s="85"/>
       <c r="EH35" s="85"/>
       <c r="EI35" s="86"/>
-      <c r="EJ35" s="84"/>
+      <c r="EJ35" s="91"/>
       <c r="EK35" s="85"/>
       <c r="EL35" s="85"/>
       <c r="EM35" s="85"/>
@@ -8443,7 +8443,7 @@
       <c r="FM35" s="36"/>
       <c r="FN35" s="36"/>
       <c r="FO35" s="36"/>
-      <c r="FP35" s="101"/>
+      <c r="FP35" s="94"/>
     </row>
     <row r="36" spans="1:172" x14ac:dyDescent="0.2">
       <c r="A36" s="42" t="s">
@@ -8465,11 +8465,11 @@
       <c r="M36" s="36"/>
       <c r="N36" s="36"/>
       <c r="O36" s="36"/>
-      <c r="P36" s="94"/>
+      <c r="P36" s="84"/>
       <c r="Q36" s="85"/>
       <c r="R36" s="85"/>
       <c r="S36" s="86"/>
-      <c r="T36" s="84"/>
+      <c r="T36" s="91"/>
       <c r="U36" s="85"/>
       <c r="V36" s="85"/>
       <c r="W36" s="85"/>
@@ -8507,11 +8507,11 @@
       <c r="BC36" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="BD36" s="94"/>
+      <c r="BD36" s="84"/>
       <c r="BE36" s="85"/>
       <c r="BF36" s="85"/>
       <c r="BG36" s="86"/>
-      <c r="BH36" s="84"/>
+      <c r="BH36" s="91"/>
       <c r="BI36" s="85"/>
       <c r="BJ36" s="85"/>
       <c r="BK36" s="85"/>
@@ -8519,7 +8519,7 @@
       <c r="BM36" s="85"/>
       <c r="BN36" s="85"/>
       <c r="BO36" s="86"/>
-      <c r="BP36" s="94"/>
+      <c r="BP36" s="84"/>
       <c r="BQ36" s="85"/>
       <c r="BR36" s="85"/>
       <c r="BS36" s="86"/>
@@ -8543,7 +8543,7 @@
       <c r="CK36" s="76"/>
       <c r="CL36" s="76"/>
       <c r="CM36" s="77"/>
-      <c r="CN36" s="84"/>
+      <c r="CN36" s="91"/>
       <c r="CO36" s="85"/>
       <c r="CP36" s="85"/>
       <c r="CQ36" s="85"/>
@@ -8587,11 +8587,11 @@
       <c r="EC36" s="36"/>
       <c r="ED36" s="36"/>
       <c r="EE36" s="36"/>
-      <c r="EF36" s="94"/>
+      <c r="EF36" s="84"/>
       <c r="EG36" s="85"/>
       <c r="EH36" s="85"/>
       <c r="EI36" s="86"/>
-      <c r="EJ36" s="84"/>
+      <c r="EJ36" s="91"/>
       <c r="EK36" s="85"/>
       <c r="EL36" s="85"/>
       <c r="EM36" s="85"/>
@@ -8623,7 +8623,7 @@
       <c r="FM36" s="36"/>
       <c r="FN36" s="36"/>
       <c r="FO36" s="36"/>
-      <c r="FP36" s="101"/>
+      <c r="FP36" s="94"/>
     </row>
     <row r="37" spans="1:172" x14ac:dyDescent="0.2">
       <c r="A37" s="42" t="s">
@@ -8645,11 +8645,11 @@
       <c r="M37" s="36"/>
       <c r="N37" s="36"/>
       <c r="O37" s="36"/>
-      <c r="P37" s="94"/>
+      <c r="P37" s="84"/>
       <c r="Q37" s="85"/>
       <c r="R37" s="85"/>
       <c r="S37" s="86"/>
-      <c r="T37" s="84"/>
+      <c r="T37" s="91"/>
       <c r="U37" s="85"/>
       <c r="V37" s="85"/>
       <c r="W37" s="85"/>
@@ -8685,11 +8685,11 @@
       <c r="BA37" s="36"/>
       <c r="BB37" s="36"/>
       <c r="BC37" s="36"/>
-      <c r="BD37" s="94"/>
+      <c r="BD37" s="84"/>
       <c r="BE37" s="85"/>
       <c r="BF37" s="85"/>
       <c r="BG37" s="86"/>
-      <c r="BH37" s="84"/>
+      <c r="BH37" s="91"/>
       <c r="BI37" s="85"/>
       <c r="BJ37" s="85"/>
       <c r="BK37" s="85"/>
@@ -8697,7 +8697,7 @@
       <c r="BM37" s="85"/>
       <c r="BN37" s="85"/>
       <c r="BO37" s="86"/>
-      <c r="BP37" s="94"/>
+      <c r="BP37" s="84"/>
       <c r="BQ37" s="85"/>
       <c r="BR37" s="85"/>
       <c r="BS37" s="86"/>
@@ -8737,7 +8737,7 @@
       <c r="CK37" s="76"/>
       <c r="CL37" s="76"/>
       <c r="CM37" s="77"/>
-      <c r="CN37" s="84"/>
+      <c r="CN37" s="91"/>
       <c r="CO37" s="85"/>
       <c r="CP37" s="85"/>
       <c r="CQ37" s="85"/>
@@ -8781,11 +8781,11 @@
       <c r="EC37" s="36"/>
       <c r="ED37" s="36"/>
       <c r="EE37" s="36"/>
-      <c r="EF37" s="94"/>
+      <c r="EF37" s="84"/>
       <c r="EG37" s="85"/>
       <c r="EH37" s="85"/>
       <c r="EI37" s="86"/>
-      <c r="EJ37" s="84"/>
+      <c r="EJ37" s="91"/>
       <c r="EK37" s="85"/>
       <c r="EL37" s="85"/>
       <c r="EM37" s="85"/>
@@ -8817,7 +8817,7 @@
       <c r="FM37" s="36"/>
       <c r="FN37" s="36"/>
       <c r="FO37" s="36"/>
-      <c r="FP37" s="101"/>
+      <c r="FP37" s="94"/>
     </row>
     <row r="38" spans="1:172" x14ac:dyDescent="0.2">
       <c r="A38" s="33"/>
@@ -8835,11 +8835,11 @@
       <c r="M38" s="36"/>
       <c r="N38" s="36"/>
       <c r="O38" s="36"/>
-      <c r="P38" s="94"/>
+      <c r="P38" s="84"/>
       <c r="Q38" s="85"/>
       <c r="R38" s="85"/>
       <c r="S38" s="86"/>
-      <c r="T38" s="84"/>
+      <c r="T38" s="91"/>
       <c r="U38" s="85"/>
       <c r="V38" s="85"/>
       <c r="W38" s="85"/>
@@ -8875,11 +8875,11 @@
       <c r="BA38" s="36"/>
       <c r="BB38" s="36"/>
       <c r="BC38" s="36"/>
-      <c r="BD38" s="94"/>
+      <c r="BD38" s="84"/>
       <c r="BE38" s="85"/>
       <c r="BF38" s="85"/>
       <c r="BG38" s="86"/>
-      <c r="BH38" s="84"/>
+      <c r="BH38" s="91"/>
       <c r="BI38" s="85"/>
       <c r="BJ38" s="85"/>
       <c r="BK38" s="85"/>
@@ -8887,7 +8887,7 @@
       <c r="BM38" s="85"/>
       <c r="BN38" s="85"/>
       <c r="BO38" s="86"/>
-      <c r="BP38" s="94"/>
+      <c r="BP38" s="84"/>
       <c r="BQ38" s="85"/>
       <c r="BR38" s="85"/>
       <c r="BS38" s="86"/>
@@ -8911,7 +8911,7 @@
       <c r="CK38" s="76"/>
       <c r="CL38" s="76"/>
       <c r="CM38" s="77"/>
-      <c r="CN38" s="84"/>
+      <c r="CN38" s="91"/>
       <c r="CO38" s="85"/>
       <c r="CP38" s="85"/>
       <c r="CQ38" s="85"/>
@@ -8955,11 +8955,11 @@
       <c r="EC38" s="36"/>
       <c r="ED38" s="36"/>
       <c r="EE38" s="36"/>
-      <c r="EF38" s="94"/>
+      <c r="EF38" s="84"/>
       <c r="EG38" s="85"/>
       <c r="EH38" s="85"/>
       <c r="EI38" s="86"/>
-      <c r="EJ38" s="84"/>
+      <c r="EJ38" s="91"/>
       <c r="EK38" s="85"/>
       <c r="EL38" s="85"/>
       <c r="EM38" s="85"/>
@@ -8991,7 +8991,7 @@
       <c r="FM38" s="36"/>
       <c r="FN38" s="36"/>
       <c r="FO38" s="36"/>
-      <c r="FP38" s="101"/>
+      <c r="FP38" s="94"/>
     </row>
     <row r="39" spans="1:172" x14ac:dyDescent="0.2">
       <c r="A39" s="43" t="s">
@@ -9013,11 +9013,11 @@
       <c r="M39" s="36"/>
       <c r="N39" s="36"/>
       <c r="O39" s="36"/>
-      <c r="P39" s="94"/>
+      <c r="P39" s="84"/>
       <c r="Q39" s="85"/>
       <c r="R39" s="85"/>
       <c r="S39" s="86"/>
-      <c r="T39" s="84"/>
+      <c r="T39" s="91"/>
       <c r="U39" s="85"/>
       <c r="V39" s="85"/>
       <c r="W39" s="85"/>
@@ -9053,11 +9053,11 @@
       <c r="BA39" s="36"/>
       <c r="BB39" s="36"/>
       <c r="BC39" s="36"/>
-      <c r="BD39" s="94"/>
+      <c r="BD39" s="84"/>
       <c r="BE39" s="85"/>
       <c r="BF39" s="85"/>
       <c r="BG39" s="86"/>
-      <c r="BH39" s="84"/>
+      <c r="BH39" s="91"/>
       <c r="BI39" s="85"/>
       <c r="BJ39" s="85"/>
       <c r="BK39" s="85"/>
@@ -9065,7 +9065,7 @@
       <c r="BM39" s="85"/>
       <c r="BN39" s="85"/>
       <c r="BO39" s="86"/>
-      <c r="BP39" s="94"/>
+      <c r="BP39" s="84"/>
       <c r="BQ39" s="85"/>
       <c r="BR39" s="85"/>
       <c r="BS39" s="86"/>
@@ -9089,7 +9089,7 @@
       <c r="CK39" s="76"/>
       <c r="CL39" s="76"/>
       <c r="CM39" s="77"/>
-      <c r="CN39" s="84"/>
+      <c r="CN39" s="91"/>
       <c r="CO39" s="85"/>
       <c r="CP39" s="85"/>
       <c r="CQ39" s="85"/>
@@ -9133,11 +9133,11 @@
       <c r="EC39" s="36"/>
       <c r="ED39" s="36"/>
       <c r="EE39" s="36"/>
-      <c r="EF39" s="94"/>
+      <c r="EF39" s="84"/>
       <c r="EG39" s="85"/>
       <c r="EH39" s="85"/>
       <c r="EI39" s="86"/>
-      <c r="EJ39" s="84"/>
+      <c r="EJ39" s="91"/>
       <c r="EK39" s="85"/>
       <c r="EL39" s="85"/>
       <c r="EM39" s="85"/>
@@ -9169,7 +9169,7 @@
       <c r="FM39" s="36"/>
       <c r="FN39" s="36"/>
       <c r="FO39" s="36"/>
-      <c r="FP39" s="101"/>
+      <c r="FP39" s="94"/>
     </row>
     <row r="40" spans="1:172" x14ac:dyDescent="0.2">
       <c r="A40" s="42" t="s">
@@ -9191,11 +9191,11 @@
       <c r="M40" s="36"/>
       <c r="N40" s="36"/>
       <c r="O40" s="36"/>
-      <c r="P40" s="94"/>
+      <c r="P40" s="84"/>
       <c r="Q40" s="85"/>
       <c r="R40" s="85"/>
       <c r="S40" s="86"/>
-      <c r="T40" s="84"/>
+      <c r="T40" s="91"/>
       <c r="U40" s="85"/>
       <c r="V40" s="85"/>
       <c r="W40" s="85"/>
@@ -9231,11 +9231,11 @@
       <c r="BA40" s="36"/>
       <c r="BB40" s="36"/>
       <c r="BC40" s="36"/>
-      <c r="BD40" s="94"/>
+      <c r="BD40" s="84"/>
       <c r="BE40" s="85"/>
       <c r="BF40" s="85"/>
       <c r="BG40" s="86"/>
-      <c r="BH40" s="84"/>
+      <c r="BH40" s="91"/>
       <c r="BI40" s="85"/>
       <c r="BJ40" s="85"/>
       <c r="BK40" s="85"/>
@@ -9243,7 +9243,7 @@
       <c r="BM40" s="85"/>
       <c r="BN40" s="85"/>
       <c r="BO40" s="86"/>
-      <c r="BP40" s="94"/>
+      <c r="BP40" s="84"/>
       <c r="BQ40" s="85"/>
       <c r="BR40" s="85"/>
       <c r="BS40" s="86"/>
@@ -9267,7 +9267,7 @@
       <c r="CK40" s="76"/>
       <c r="CL40" s="76"/>
       <c r="CM40" s="77"/>
-      <c r="CN40" s="84"/>
+      <c r="CN40" s="91"/>
       <c r="CO40" s="85"/>
       <c r="CP40" s="85"/>
       <c r="CQ40" s="85"/>
@@ -9315,11 +9315,11 @@
       <c r="EC40" s="36"/>
       <c r="ED40" s="36"/>
       <c r="EE40" s="36"/>
-      <c r="EF40" s="94"/>
+      <c r="EF40" s="84"/>
       <c r="EG40" s="85"/>
       <c r="EH40" s="85"/>
       <c r="EI40" s="86"/>
-      <c r="EJ40" s="84"/>
+      <c r="EJ40" s="91"/>
       <c r="EK40" s="85"/>
       <c r="EL40" s="85"/>
       <c r="EM40" s="85"/>
@@ -9351,7 +9351,7 @@
       <c r="FM40" s="36"/>
       <c r="FN40" s="36"/>
       <c r="FO40" s="36"/>
-      <c r="FP40" s="101"/>
+      <c r="FP40" s="94"/>
     </row>
     <row r="41" spans="1:172" x14ac:dyDescent="0.2">
       <c r="A41" s="42" t="s">
@@ -9373,11 +9373,11 @@
       <c r="M41" s="36"/>
       <c r="N41" s="36"/>
       <c r="O41" s="36"/>
-      <c r="P41" s="94"/>
+      <c r="P41" s="84"/>
       <c r="Q41" s="85"/>
       <c r="R41" s="85"/>
       <c r="S41" s="86"/>
-      <c r="T41" s="84"/>
+      <c r="T41" s="91"/>
       <c r="U41" s="85"/>
       <c r="V41" s="85"/>
       <c r="W41" s="85"/>
@@ -9413,11 +9413,11 @@
       <c r="BA41" s="36"/>
       <c r="BB41" s="36"/>
       <c r="BC41" s="36"/>
-      <c r="BD41" s="94"/>
+      <c r="BD41" s="84"/>
       <c r="BE41" s="85"/>
       <c r="BF41" s="85"/>
       <c r="BG41" s="86"/>
-      <c r="BH41" s="84"/>
+      <c r="BH41" s="91"/>
       <c r="BI41" s="85"/>
       <c r="BJ41" s="85"/>
       <c r="BK41" s="85"/>
@@ -9425,7 +9425,7 @@
       <c r="BM41" s="85"/>
       <c r="BN41" s="85"/>
       <c r="BO41" s="86"/>
-      <c r="BP41" s="94"/>
+      <c r="BP41" s="84"/>
       <c r="BQ41" s="85"/>
       <c r="BR41" s="85"/>
       <c r="BS41" s="86"/>
@@ -9449,7 +9449,7 @@
       <c r="CK41" s="76"/>
       <c r="CL41" s="76"/>
       <c r="CM41" s="77"/>
-      <c r="CN41" s="84"/>
+      <c r="CN41" s="91"/>
       <c r="CO41" s="85"/>
       <c r="CP41" s="85"/>
       <c r="CQ41" s="85"/>
@@ -9497,11 +9497,11 @@
       <c r="EC41" s="36"/>
       <c r="ED41" s="36"/>
       <c r="EE41" s="36"/>
-      <c r="EF41" s="94"/>
+      <c r="EF41" s="84"/>
       <c r="EG41" s="85"/>
       <c r="EH41" s="85"/>
       <c r="EI41" s="86"/>
-      <c r="EJ41" s="84"/>
+      <c r="EJ41" s="91"/>
       <c r="EK41" s="85"/>
       <c r="EL41" s="85"/>
       <c r="EM41" s="85"/>
@@ -9533,7 +9533,7 @@
       <c r="FM41" s="36"/>
       <c r="FN41" s="36"/>
       <c r="FO41" s="36"/>
-      <c r="FP41" s="101"/>
+      <c r="FP41" s="94"/>
     </row>
     <row r="42" spans="1:172" x14ac:dyDescent="0.2">
       <c r="A42" s="42" t="s">
@@ -9555,11 +9555,11 @@
       <c r="M42" s="36"/>
       <c r="N42" s="36"/>
       <c r="O42" s="36"/>
-      <c r="P42" s="94"/>
+      <c r="P42" s="84"/>
       <c r="Q42" s="85"/>
       <c r="R42" s="85"/>
       <c r="S42" s="86"/>
-      <c r="T42" s="84"/>
+      <c r="T42" s="91"/>
       <c r="U42" s="85"/>
       <c r="V42" s="85"/>
       <c r="W42" s="85"/>
@@ -9595,11 +9595,11 @@
       <c r="BA42" s="36"/>
       <c r="BB42" s="36"/>
       <c r="BC42" s="36"/>
-      <c r="BD42" s="94"/>
+      <c r="BD42" s="84"/>
       <c r="BE42" s="85"/>
       <c r="BF42" s="85"/>
       <c r="BG42" s="86"/>
-      <c r="BH42" s="84"/>
+      <c r="BH42" s="91"/>
       <c r="BI42" s="85"/>
       <c r="BJ42" s="85"/>
       <c r="BK42" s="85"/>
@@ -9607,7 +9607,7 @@
       <c r="BM42" s="85"/>
       <c r="BN42" s="85"/>
       <c r="BO42" s="86"/>
-      <c r="BP42" s="94"/>
+      <c r="BP42" s="84"/>
       <c r="BQ42" s="85"/>
       <c r="BR42" s="85"/>
       <c r="BS42" s="86"/>
@@ -9631,7 +9631,7 @@
       <c r="CK42" s="76"/>
       <c r="CL42" s="76"/>
       <c r="CM42" s="77"/>
-      <c r="CN42" s="84"/>
+      <c r="CN42" s="91"/>
       <c r="CO42" s="85"/>
       <c r="CP42" s="85"/>
       <c r="CQ42" s="85"/>
@@ -9679,11 +9679,11 @@
       <c r="EC42" s="36"/>
       <c r="ED42" s="36"/>
       <c r="EE42" s="36"/>
-      <c r="EF42" s="94"/>
+      <c r="EF42" s="84"/>
       <c r="EG42" s="85"/>
       <c r="EH42" s="85"/>
       <c r="EI42" s="86"/>
-      <c r="EJ42" s="84"/>
+      <c r="EJ42" s="91"/>
       <c r="EK42" s="85"/>
       <c r="EL42" s="85"/>
       <c r="EM42" s="85"/>
@@ -9715,7 +9715,7 @@
       <c r="FM42" s="36"/>
       <c r="FN42" s="36"/>
       <c r="FO42" s="36"/>
-      <c r="FP42" s="101"/>
+      <c r="FP42" s="94"/>
     </row>
     <row r="43" spans="1:172" x14ac:dyDescent="0.2">
       <c r="A43" s="42" t="s">
@@ -9737,11 +9737,11 @@
       <c r="M43" s="36"/>
       <c r="N43" s="36"/>
       <c r="O43" s="36"/>
-      <c r="P43" s="94"/>
+      <c r="P43" s="84"/>
       <c r="Q43" s="85"/>
       <c r="R43" s="85"/>
       <c r="S43" s="86"/>
-      <c r="T43" s="84"/>
+      <c r="T43" s="91"/>
       <c r="U43" s="85"/>
       <c r="V43" s="85"/>
       <c r="W43" s="85"/>
@@ -9777,11 +9777,11 @@
       <c r="BA43" s="36"/>
       <c r="BB43" s="36"/>
       <c r="BC43" s="36"/>
-      <c r="BD43" s="94"/>
+      <c r="BD43" s="84"/>
       <c r="BE43" s="85"/>
       <c r="BF43" s="85"/>
       <c r="BG43" s="86"/>
-      <c r="BH43" s="84"/>
+      <c r="BH43" s="91"/>
       <c r="BI43" s="85"/>
       <c r="BJ43" s="85"/>
       <c r="BK43" s="85"/>
@@ -9789,7 +9789,7 @@
       <c r="BM43" s="85"/>
       <c r="BN43" s="85"/>
       <c r="BO43" s="86"/>
-      <c r="BP43" s="94"/>
+      <c r="BP43" s="84"/>
       <c r="BQ43" s="85"/>
       <c r="BR43" s="85"/>
       <c r="BS43" s="86"/>
@@ -9813,7 +9813,7 @@
       <c r="CK43" s="76"/>
       <c r="CL43" s="76"/>
       <c r="CM43" s="77"/>
-      <c r="CN43" s="84"/>
+      <c r="CN43" s="91"/>
       <c r="CO43" s="85"/>
       <c r="CP43" s="85"/>
       <c r="CQ43" s="85"/>
@@ -9859,11 +9859,11 @@
       <c r="EC43" s="36"/>
       <c r="ED43" s="36"/>
       <c r="EE43" s="36"/>
-      <c r="EF43" s="94"/>
+      <c r="EF43" s="84"/>
       <c r="EG43" s="85"/>
       <c r="EH43" s="85"/>
       <c r="EI43" s="86"/>
-      <c r="EJ43" s="84"/>
+      <c r="EJ43" s="91"/>
       <c r="EK43" s="85"/>
       <c r="EL43" s="85"/>
       <c r="EM43" s="85"/>
@@ -9895,7 +9895,7 @@
       <c r="FM43" s="36"/>
       <c r="FN43" s="36"/>
       <c r="FO43" s="36"/>
-      <c r="FP43" s="101"/>
+      <c r="FP43" s="94"/>
     </row>
     <row r="44" spans="1:172" x14ac:dyDescent="0.2">
       <c r="A44" s="42" t="s">
@@ -9917,11 +9917,11 @@
       <c r="M44" s="36"/>
       <c r="N44" s="36"/>
       <c r="O44" s="36"/>
-      <c r="P44" s="94"/>
+      <c r="P44" s="84"/>
       <c r="Q44" s="85"/>
       <c r="R44" s="85"/>
       <c r="S44" s="86"/>
-      <c r="T44" s="84"/>
+      <c r="T44" s="91"/>
       <c r="U44" s="85"/>
       <c r="V44" s="85"/>
       <c r="W44" s="85"/>
@@ -9957,11 +9957,11 @@
       <c r="BA44" s="36"/>
       <c r="BB44" s="36"/>
       <c r="BC44" s="36"/>
-      <c r="BD44" s="94"/>
+      <c r="BD44" s="84"/>
       <c r="BE44" s="85"/>
       <c r="BF44" s="85"/>
       <c r="BG44" s="86"/>
-      <c r="BH44" s="84"/>
+      <c r="BH44" s="91"/>
       <c r="BI44" s="85"/>
       <c r="BJ44" s="85"/>
       <c r="BK44" s="85"/>
@@ -9969,7 +9969,7 @@
       <c r="BM44" s="85"/>
       <c r="BN44" s="85"/>
       <c r="BO44" s="86"/>
-      <c r="BP44" s="94"/>
+      <c r="BP44" s="84"/>
       <c r="BQ44" s="85"/>
       <c r="BR44" s="85"/>
       <c r="BS44" s="86"/>
@@ -9993,7 +9993,7 @@
       <c r="CK44" s="76"/>
       <c r="CL44" s="76"/>
       <c r="CM44" s="77"/>
-      <c r="CN44" s="84"/>
+      <c r="CN44" s="91"/>
       <c r="CO44" s="85"/>
       <c r="CP44" s="85"/>
       <c r="CQ44" s="85"/>
@@ -10039,11 +10039,11 @@
       <c r="EC44" s="36"/>
       <c r="ED44" s="36"/>
       <c r="EE44" s="36"/>
-      <c r="EF44" s="94"/>
+      <c r="EF44" s="84"/>
       <c r="EG44" s="85"/>
       <c r="EH44" s="85"/>
       <c r="EI44" s="86"/>
-      <c r="EJ44" s="84"/>
+      <c r="EJ44" s="91"/>
       <c r="EK44" s="85"/>
       <c r="EL44" s="85"/>
       <c r="EM44" s="85"/>
@@ -10075,7 +10075,7 @@
       <c r="FM44" s="36"/>
       <c r="FN44" s="36"/>
       <c r="FO44" s="36"/>
-      <c r="FP44" s="101"/>
+      <c r="FP44" s="94"/>
     </row>
     <row r="45" spans="1:172" x14ac:dyDescent="0.2">
       <c r="A45" s="42" t="s">
@@ -10097,11 +10097,11 @@
       <c r="M45" s="36"/>
       <c r="N45" s="36"/>
       <c r="O45" s="36"/>
-      <c r="P45" s="94"/>
+      <c r="P45" s="84"/>
       <c r="Q45" s="85"/>
       <c r="R45" s="85"/>
       <c r="S45" s="86"/>
-      <c r="T45" s="84"/>
+      <c r="T45" s="91"/>
       <c r="U45" s="85"/>
       <c r="V45" s="85"/>
       <c r="W45" s="85"/>
@@ -10137,11 +10137,11 @@
       <c r="BA45" s="36"/>
       <c r="BB45" s="36"/>
       <c r="BC45" s="36"/>
-      <c r="BD45" s="94"/>
+      <c r="BD45" s="84"/>
       <c r="BE45" s="85"/>
       <c r="BF45" s="85"/>
       <c r="BG45" s="86"/>
-      <c r="BH45" s="84"/>
+      <c r="BH45" s="91"/>
       <c r="BI45" s="85"/>
       <c r="BJ45" s="85"/>
       <c r="BK45" s="85"/>
@@ -10149,7 +10149,7 @@
       <c r="BM45" s="85"/>
       <c r="BN45" s="85"/>
       <c r="BO45" s="86"/>
-      <c r="BP45" s="94"/>
+      <c r="BP45" s="84"/>
       <c r="BQ45" s="85"/>
       <c r="BR45" s="85"/>
       <c r="BS45" s="86"/>
@@ -10173,7 +10173,7 @@
       <c r="CK45" s="76"/>
       <c r="CL45" s="76"/>
       <c r="CM45" s="77"/>
-      <c r="CN45" s="84"/>
+      <c r="CN45" s="91"/>
       <c r="CO45" s="85"/>
       <c r="CP45" s="85"/>
       <c r="CQ45" s="85"/>
@@ -10219,11 +10219,11 @@
       <c r="EC45" s="58"/>
       <c r="ED45" s="36"/>
       <c r="EE45" s="36"/>
-      <c r="EF45" s="94"/>
+      <c r="EF45" s="84"/>
       <c r="EG45" s="85"/>
       <c r="EH45" s="85"/>
       <c r="EI45" s="86"/>
-      <c r="EJ45" s="84"/>
+      <c r="EJ45" s="91"/>
       <c r="EK45" s="85"/>
       <c r="EL45" s="85"/>
       <c r="EM45" s="85"/>
@@ -10255,7 +10255,7 @@
       <c r="FM45" s="36"/>
       <c r="FN45" s="36"/>
       <c r="FO45" s="36"/>
-      <c r="FP45" s="101"/>
+      <c r="FP45" s="94"/>
     </row>
     <row r="46" spans="1:172" x14ac:dyDescent="0.2">
       <c r="A46" s="42" t="s">
@@ -10277,11 +10277,11 @@
       <c r="M46" s="36"/>
       <c r="N46" s="36"/>
       <c r="O46" s="36"/>
-      <c r="P46" s="94"/>
+      <c r="P46" s="84"/>
       <c r="Q46" s="85"/>
       <c r="R46" s="85"/>
       <c r="S46" s="86"/>
-      <c r="T46" s="84"/>
+      <c r="T46" s="91"/>
       <c r="U46" s="85"/>
       <c r="V46" s="85"/>
       <c r="W46" s="85"/>
@@ -10317,11 +10317,11 @@
       <c r="BA46" s="36"/>
       <c r="BB46" s="36"/>
       <c r="BC46" s="36"/>
-      <c r="BD46" s="94"/>
+      <c r="BD46" s="84"/>
       <c r="BE46" s="85"/>
       <c r="BF46" s="85"/>
       <c r="BG46" s="86"/>
-      <c r="BH46" s="84"/>
+      <c r="BH46" s="91"/>
       <c r="BI46" s="85"/>
       <c r="BJ46" s="85"/>
       <c r="BK46" s="85"/>
@@ -10329,7 +10329,7 @@
       <c r="BM46" s="85"/>
       <c r="BN46" s="85"/>
       <c r="BO46" s="86"/>
-      <c r="BP46" s="94"/>
+      <c r="BP46" s="84"/>
       <c r="BQ46" s="85"/>
       <c r="BR46" s="85"/>
       <c r="BS46" s="86"/>
@@ -10353,7 +10353,7 @@
       <c r="CK46" s="76"/>
       <c r="CL46" s="76"/>
       <c r="CM46" s="77"/>
-      <c r="CN46" s="84"/>
+      <c r="CN46" s="91"/>
       <c r="CO46" s="85"/>
       <c r="CP46" s="85"/>
       <c r="CQ46" s="85"/>
@@ -10399,11 +10399,11 @@
       <c r="EC46" s="36"/>
       <c r="ED46" s="58"/>
       <c r="EE46" s="58"/>
-      <c r="EF46" s="94"/>
+      <c r="EF46" s="84"/>
       <c r="EG46" s="85"/>
       <c r="EH46" s="85"/>
       <c r="EI46" s="86"/>
-      <c r="EJ46" s="84"/>
+      <c r="EJ46" s="91"/>
       <c r="EK46" s="85"/>
       <c r="EL46" s="85"/>
       <c r="EM46" s="85"/>
@@ -10435,7 +10435,7 @@
       <c r="FM46" s="36"/>
       <c r="FN46" s="36"/>
       <c r="FO46" s="36"/>
-      <c r="FP46" s="101"/>
+      <c r="FP46" s="94"/>
     </row>
     <row r="47" spans="1:172" x14ac:dyDescent="0.2">
       <c r="A47" s="42"/>
@@ -10453,11 +10453,11 @@
       <c r="M47" s="36"/>
       <c r="N47" s="36"/>
       <c r="O47" s="36"/>
-      <c r="P47" s="94"/>
+      <c r="P47" s="84"/>
       <c r="Q47" s="85"/>
       <c r="R47" s="85"/>
       <c r="S47" s="86"/>
-      <c r="T47" s="84"/>
+      <c r="T47" s="91"/>
       <c r="U47" s="85"/>
       <c r="V47" s="85"/>
       <c r="W47" s="85"/>
@@ -10493,11 +10493,11 @@
       <c r="BA47" s="36"/>
       <c r="BB47" s="36"/>
       <c r="BC47" s="36"/>
-      <c r="BD47" s="94"/>
+      <c r="BD47" s="84"/>
       <c r="BE47" s="85"/>
       <c r="BF47" s="85"/>
       <c r="BG47" s="86"/>
-      <c r="BH47" s="84"/>
+      <c r="BH47" s="91"/>
       <c r="BI47" s="85"/>
       <c r="BJ47" s="85"/>
       <c r="BK47" s="85"/>
@@ -10505,7 +10505,7 @@
       <c r="BM47" s="85"/>
       <c r="BN47" s="85"/>
       <c r="BO47" s="86"/>
-      <c r="BP47" s="94"/>
+      <c r="BP47" s="84"/>
       <c r="BQ47" s="85"/>
       <c r="BR47" s="85"/>
       <c r="BS47" s="86"/>
@@ -10529,7 +10529,7 @@
       <c r="CK47" s="76"/>
       <c r="CL47" s="76"/>
       <c r="CM47" s="77"/>
-      <c r="CN47" s="84"/>
+      <c r="CN47" s="91"/>
       <c r="CO47" s="85"/>
       <c r="CP47" s="85"/>
       <c r="CQ47" s="85"/>
@@ -10573,11 +10573,11 @@
       <c r="EC47" s="36"/>
       <c r="ED47" s="36"/>
       <c r="EE47" s="36"/>
-      <c r="EF47" s="94"/>
+      <c r="EF47" s="84"/>
       <c r="EG47" s="85"/>
       <c r="EH47" s="85"/>
       <c r="EI47" s="86"/>
-      <c r="EJ47" s="84"/>
+      <c r="EJ47" s="91"/>
       <c r="EK47" s="85"/>
       <c r="EL47" s="85"/>
       <c r="EM47" s="85"/>
@@ -10609,7 +10609,7 @@
       <c r="FM47" s="36"/>
       <c r="FN47" s="36"/>
       <c r="FO47" s="36"/>
-      <c r="FP47" s="101"/>
+      <c r="FP47" s="94"/>
     </row>
     <row r="48" spans="1:172" x14ac:dyDescent="0.2">
       <c r="A48" s="48" t="s">
@@ -10631,11 +10631,11 @@
       <c r="M48" s="36"/>
       <c r="N48" s="36"/>
       <c r="O48" s="36"/>
-      <c r="P48" s="94"/>
+      <c r="P48" s="84"/>
       <c r="Q48" s="85"/>
       <c r="R48" s="85"/>
       <c r="S48" s="86"/>
-      <c r="T48" s="84"/>
+      <c r="T48" s="91"/>
       <c r="U48" s="85"/>
       <c r="V48" s="85"/>
       <c r="W48" s="85"/>
@@ -10671,11 +10671,11 @@
       <c r="BA48" s="36"/>
       <c r="BB48" s="36"/>
       <c r="BC48" s="36"/>
-      <c r="BD48" s="94"/>
+      <c r="BD48" s="84"/>
       <c r="BE48" s="85"/>
       <c r="BF48" s="85"/>
       <c r="BG48" s="86"/>
-      <c r="BH48" s="84"/>
+      <c r="BH48" s="91"/>
       <c r="BI48" s="85"/>
       <c r="BJ48" s="85"/>
       <c r="BK48" s="85"/>
@@ -10683,7 +10683,7 @@
       <c r="BM48" s="85"/>
       <c r="BN48" s="85"/>
       <c r="BO48" s="86"/>
-      <c r="BP48" s="94"/>
+      <c r="BP48" s="84"/>
       <c r="BQ48" s="85"/>
       <c r="BR48" s="85"/>
       <c r="BS48" s="86"/>
@@ -10707,7 +10707,7 @@
       <c r="CK48" s="76"/>
       <c r="CL48" s="76"/>
       <c r="CM48" s="77"/>
-      <c r="CN48" s="84"/>
+      <c r="CN48" s="91"/>
       <c r="CO48" s="85"/>
       <c r="CP48" s="85"/>
       <c r="CQ48" s="85"/>
@@ -10751,11 +10751,11 @@
       <c r="EC48" s="36"/>
       <c r="ED48" s="36"/>
       <c r="EE48" s="36"/>
-      <c r="EF48" s="94"/>
+      <c r="EF48" s="84"/>
       <c r="EG48" s="85"/>
       <c r="EH48" s="85"/>
       <c r="EI48" s="86"/>
-      <c r="EJ48" s="84"/>
+      <c r="EJ48" s="91"/>
       <c r="EK48" s="85"/>
       <c r="EL48" s="85"/>
       <c r="EM48" s="85"/>
@@ -10787,7 +10787,7 @@
       <c r="FM48" s="36"/>
       <c r="FN48" s="36"/>
       <c r="FO48" s="36"/>
-      <c r="FP48" s="101"/>
+      <c r="FP48" s="94"/>
     </row>
     <row r="49" spans="1:172" x14ac:dyDescent="0.2">
       <c r="A49" s="42" t="s">
@@ -10809,11 +10809,11 @@
       <c r="M49" s="36"/>
       <c r="N49" s="36"/>
       <c r="O49" s="36"/>
-      <c r="P49" s="94"/>
+      <c r="P49" s="84"/>
       <c r="Q49" s="85"/>
       <c r="R49" s="85"/>
       <c r="S49" s="86"/>
-      <c r="T49" s="84"/>
+      <c r="T49" s="91"/>
       <c r="U49" s="85"/>
       <c r="V49" s="85"/>
       <c r="W49" s="85"/>
@@ -10849,11 +10849,11 @@
       <c r="BA49" s="36"/>
       <c r="BB49" s="36"/>
       <c r="BC49" s="36"/>
-      <c r="BD49" s="94"/>
+      <c r="BD49" s="84"/>
       <c r="BE49" s="85"/>
       <c r="BF49" s="85"/>
       <c r="BG49" s="86"/>
-      <c r="BH49" s="84"/>
+      <c r="BH49" s="91"/>
       <c r="BI49" s="85"/>
       <c r="BJ49" s="85"/>
       <c r="BK49" s="85"/>
@@ -10861,7 +10861,7 @@
       <c r="BM49" s="85"/>
       <c r="BN49" s="85"/>
       <c r="BO49" s="86"/>
-      <c r="BP49" s="94"/>
+      <c r="BP49" s="84"/>
       <c r="BQ49" s="85"/>
       <c r="BR49" s="85"/>
       <c r="BS49" s="86"/>
@@ -10885,7 +10885,7 @@
       <c r="CK49" s="76"/>
       <c r="CL49" s="76"/>
       <c r="CM49" s="77"/>
-      <c r="CN49" s="84"/>
+      <c r="CN49" s="91"/>
       <c r="CO49" s="85"/>
       <c r="CP49" s="85"/>
       <c r="CQ49" s="85"/>
@@ -10931,11 +10931,11 @@
       <c r="EC49" s="36"/>
       <c r="ED49" s="36"/>
       <c r="EE49" s="36"/>
-      <c r="EF49" s="94"/>
+      <c r="EF49" s="84"/>
       <c r="EG49" s="85"/>
       <c r="EH49" s="85"/>
       <c r="EI49" s="86"/>
-      <c r="EJ49" s="84"/>
+      <c r="EJ49" s="91"/>
       <c r="EK49" s="85"/>
       <c r="EL49" s="85"/>
       <c r="EM49" s="85"/>
@@ -10967,7 +10967,7 @@
       <c r="FM49" s="36"/>
       <c r="FN49" s="36"/>
       <c r="FO49" s="36"/>
-      <c r="FP49" s="101"/>
+      <c r="FP49" s="94"/>
     </row>
     <row r="50" spans="1:172" x14ac:dyDescent="0.2">
       <c r="A50" s="42" t="s">
@@ -10989,11 +10989,11 @@
       <c r="M50" s="36"/>
       <c r="N50" s="36"/>
       <c r="O50" s="36"/>
-      <c r="P50" s="94"/>
+      <c r="P50" s="84"/>
       <c r="Q50" s="85"/>
       <c r="R50" s="85"/>
       <c r="S50" s="86"/>
-      <c r="T50" s="84"/>
+      <c r="T50" s="91"/>
       <c r="U50" s="85"/>
       <c r="V50" s="85"/>
       <c r="W50" s="85"/>
@@ -11029,11 +11029,11 @@
       <c r="BA50" s="36"/>
       <c r="BB50" s="36"/>
       <c r="BC50" s="36"/>
-      <c r="BD50" s="94"/>
+      <c r="BD50" s="84"/>
       <c r="BE50" s="85"/>
       <c r="BF50" s="85"/>
       <c r="BG50" s="86"/>
-      <c r="BH50" s="84"/>
+      <c r="BH50" s="91"/>
       <c r="BI50" s="85"/>
       <c r="BJ50" s="85"/>
       <c r="BK50" s="85"/>
@@ -11041,7 +11041,7 @@
       <c r="BM50" s="85"/>
       <c r="BN50" s="85"/>
       <c r="BO50" s="86"/>
-      <c r="BP50" s="94"/>
+      <c r="BP50" s="84"/>
       <c r="BQ50" s="85"/>
       <c r="BR50" s="85"/>
       <c r="BS50" s="86"/>
@@ -11065,7 +11065,7 @@
       <c r="CK50" s="76"/>
       <c r="CL50" s="76"/>
       <c r="CM50" s="77"/>
-      <c r="CN50" s="84"/>
+      <c r="CN50" s="91"/>
       <c r="CO50" s="85"/>
       <c r="CP50" s="85"/>
       <c r="CQ50" s="85"/>
@@ -11111,11 +11111,11 @@
       <c r="EC50" s="36"/>
       <c r="ED50" s="36"/>
       <c r="EE50" s="36"/>
-      <c r="EF50" s="94"/>
+      <c r="EF50" s="84"/>
       <c r="EG50" s="85"/>
       <c r="EH50" s="85"/>
       <c r="EI50" s="86"/>
-      <c r="EJ50" s="84"/>
+      <c r="EJ50" s="91"/>
       <c r="EK50" s="85"/>
       <c r="EL50" s="85"/>
       <c r="EM50" s="85"/>
@@ -11146,13 +11146,15 @@
       <c r="FM50" s="36"/>
       <c r="FN50" s="36"/>
       <c r="FO50" s="36"/>
-      <c r="FP50" s="101"/>
+      <c r="FP50" s="94"/>
     </row>
     <row r="51" spans="1:172" x14ac:dyDescent="0.2">
       <c r="A51" s="42" t="s">
         <v>50</v>
       </c>
-      <c r="B51" s="34"/>
+      <c r="B51" s="34" t="s">
+        <v>63</v>
+      </c>
       <c r="C51" s="13"/>
       <c r="D51" s="36"/>
       <c r="E51" s="36"/>
@@ -11166,11 +11168,11 @@
       <c r="M51" s="36"/>
       <c r="N51" s="36"/>
       <c r="O51" s="36"/>
-      <c r="P51" s="94"/>
+      <c r="P51" s="84"/>
       <c r="Q51" s="85"/>
       <c r="R51" s="85"/>
       <c r="S51" s="86"/>
-      <c r="T51" s="84"/>
+      <c r="T51" s="91"/>
       <c r="U51" s="85"/>
       <c r="V51" s="85"/>
       <c r="W51" s="85"/>
@@ -11206,11 +11208,11 @@
       <c r="BA51" s="50"/>
       <c r="BB51" s="50"/>
       <c r="BC51" s="50"/>
-      <c r="BD51" s="94"/>
+      <c r="BD51" s="84"/>
       <c r="BE51" s="85"/>
       <c r="BF51" s="85"/>
       <c r="BG51" s="86"/>
-      <c r="BH51" s="84"/>
+      <c r="BH51" s="91"/>
       <c r="BI51" s="85"/>
       <c r="BJ51" s="85"/>
       <c r="BK51" s="85"/>
@@ -11218,7 +11220,7 @@
       <c r="BM51" s="85"/>
       <c r="BN51" s="85"/>
       <c r="BO51" s="86"/>
-      <c r="BP51" s="94"/>
+      <c r="BP51" s="84"/>
       <c r="BQ51" s="85"/>
       <c r="BR51" s="85"/>
       <c r="BS51" s="86"/>
@@ -11242,7 +11244,7 @@
       <c r="CK51" s="76"/>
       <c r="CL51" s="76"/>
       <c r="CM51" s="77"/>
-      <c r="CN51" s="84"/>
+      <c r="CN51" s="91"/>
       <c r="CO51" s="85"/>
       <c r="CP51" s="85"/>
       <c r="CQ51" s="85"/>
@@ -11282,17 +11284,29 @@
       </c>
       <c r="DX51" s="50"/>
       <c r="DY51" s="50"/>
-      <c r="DZ51" s="50"/>
-      <c r="EA51" s="50"/>
-      <c r="EB51" s="50"/>
-      <c r="EC51" s="50"/>
-      <c r="ED51" s="50"/>
-      <c r="EE51" s="50"/>
-      <c r="EF51" s="94"/>
+      <c r="DZ51" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="EA51" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="EB51" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="EC51" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="ED51" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="EE51" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="EF51" s="84"/>
       <c r="EG51" s="85"/>
       <c r="EH51" s="85"/>
       <c r="EI51" s="86"/>
-      <c r="EJ51" s="84"/>
+      <c r="EJ51" s="91"/>
       <c r="EK51" s="85"/>
       <c r="EL51" s="85"/>
       <c r="EM51" s="85"/>
@@ -11308,14 +11322,30 @@
       <c r="EW51" s="76"/>
       <c r="EX51" s="76"/>
       <c r="EY51" s="77"/>
-      <c r="EZ51" s="50"/>
-      <c r="FA51" s="50"/>
-      <c r="FB51" s="50"/>
-      <c r="FC51" s="50"/>
-      <c r="FD51" s="50"/>
-      <c r="FE51" s="50"/>
-      <c r="FF51" s="50"/>
-      <c r="FG51" s="50"/>
+      <c r="EZ51" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="FA51" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="FB51" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="FC51" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="FD51" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="FE51" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="FF51" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="FG51" s="50" t="s">
+        <v>46</v>
+      </c>
       <c r="FH51" s="35"/>
       <c r="FI51" s="36"/>
       <c r="FJ51" s="36"/>
@@ -11324,7 +11354,7 @@
       <c r="FM51" s="36"/>
       <c r="FN51" s="36"/>
       <c r="FO51" s="36"/>
-      <c r="FP51" s="101"/>
+      <c r="FP51" s="94"/>
     </row>
     <row r="52" spans="1:172" x14ac:dyDescent="0.2">
       <c r="A52" s="33"/>
@@ -11342,11 +11372,11 @@
       <c r="M52" s="36"/>
       <c r="N52" s="36"/>
       <c r="O52" s="36"/>
-      <c r="P52" s="94"/>
+      <c r="P52" s="84"/>
       <c r="Q52" s="85"/>
       <c r="R52" s="85"/>
       <c r="S52" s="86"/>
-      <c r="T52" s="84"/>
+      <c r="T52" s="91"/>
       <c r="U52" s="85"/>
       <c r="V52" s="85"/>
       <c r="W52" s="85"/>
@@ -11382,11 +11412,11 @@
       <c r="BA52" s="36"/>
       <c r="BB52" s="36"/>
       <c r="BC52" s="36"/>
-      <c r="BD52" s="94"/>
+      <c r="BD52" s="84"/>
       <c r="BE52" s="85"/>
       <c r="BF52" s="85"/>
       <c r="BG52" s="86"/>
-      <c r="BH52" s="84"/>
+      <c r="BH52" s="91"/>
       <c r="BI52" s="85"/>
       <c r="BJ52" s="85"/>
       <c r="BK52" s="85"/>
@@ -11394,7 +11424,7 @@
       <c r="BM52" s="85"/>
       <c r="BN52" s="85"/>
       <c r="BO52" s="86"/>
-      <c r="BP52" s="94"/>
+      <c r="BP52" s="84"/>
       <c r="BQ52" s="85"/>
       <c r="BR52" s="85"/>
       <c r="BS52" s="86"/>
@@ -11418,7 +11448,7 @@
       <c r="CK52" s="76"/>
       <c r="CL52" s="76"/>
       <c r="CM52" s="77"/>
-      <c r="CN52" s="84"/>
+      <c r="CN52" s="91"/>
       <c r="CO52" s="85"/>
       <c r="CP52" s="85"/>
       <c r="CQ52" s="85"/>
@@ -11462,11 +11492,11 @@
       <c r="EC52" s="36"/>
       <c r="ED52" s="36"/>
       <c r="EE52" s="36"/>
-      <c r="EF52" s="94"/>
+      <c r="EF52" s="84"/>
       <c r="EG52" s="85"/>
       <c r="EH52" s="85"/>
       <c r="EI52" s="86"/>
-      <c r="EJ52" s="84"/>
+      <c r="EJ52" s="91"/>
       <c r="EK52" s="85"/>
       <c r="EL52" s="85"/>
       <c r="EM52" s="85"/>
@@ -11498,7 +11528,7 @@
       <c r="FM52" s="36"/>
       <c r="FN52" s="36"/>
       <c r="FO52" s="36"/>
-      <c r="FP52" s="101"/>
+      <c r="FP52" s="94"/>
     </row>
     <row r="53" spans="1:172" x14ac:dyDescent="0.2">
       <c r="A53" s="33"/>
@@ -11516,11 +11546,11 @@
       <c r="M53" s="36"/>
       <c r="N53" s="36"/>
       <c r="O53" s="36"/>
-      <c r="P53" s="94"/>
+      <c r="P53" s="84"/>
       <c r="Q53" s="85"/>
       <c r="R53" s="85"/>
       <c r="S53" s="86"/>
-      <c r="T53" s="84"/>
+      <c r="T53" s="91"/>
       <c r="U53" s="85"/>
       <c r="V53" s="85"/>
       <c r="W53" s="85"/>
@@ -11556,11 +11586,11 @@
       <c r="BA53" s="36"/>
       <c r="BB53" s="36"/>
       <c r="BC53" s="36"/>
-      <c r="BD53" s="94"/>
+      <c r="BD53" s="84"/>
       <c r="BE53" s="85"/>
       <c r="BF53" s="85"/>
       <c r="BG53" s="86"/>
-      <c r="BH53" s="84"/>
+      <c r="BH53" s="91"/>
       <c r="BI53" s="85"/>
       <c r="BJ53" s="85"/>
       <c r="BK53" s="85"/>
@@ -11568,7 +11598,7 @@
       <c r="BM53" s="85"/>
       <c r="BN53" s="85"/>
       <c r="BO53" s="86"/>
-      <c r="BP53" s="94"/>
+      <c r="BP53" s="84"/>
       <c r="BQ53" s="85"/>
       <c r="BR53" s="85"/>
       <c r="BS53" s="86"/>
@@ -11592,7 +11622,7 @@
       <c r="CK53" s="76"/>
       <c r="CL53" s="76"/>
       <c r="CM53" s="77"/>
-      <c r="CN53" s="84"/>
+      <c r="CN53" s="91"/>
       <c r="CO53" s="85"/>
       <c r="CP53" s="85"/>
       <c r="CQ53" s="85"/>
@@ -11636,11 +11666,11 @@
       <c r="EC53" s="36"/>
       <c r="ED53" s="36"/>
       <c r="EE53" s="36"/>
-      <c r="EF53" s="94"/>
+      <c r="EF53" s="84"/>
       <c r="EG53" s="85"/>
       <c r="EH53" s="85"/>
       <c r="EI53" s="86"/>
-      <c r="EJ53" s="84"/>
+      <c r="EJ53" s="91"/>
       <c r="EK53" s="85"/>
       <c r="EL53" s="85"/>
       <c r="EM53" s="85"/>
@@ -11672,7 +11702,7 @@
       <c r="FM53" s="36"/>
       <c r="FN53" s="36"/>
       <c r="FO53" s="36"/>
-      <c r="FP53" s="101"/>
+      <c r="FP53" s="94"/>
     </row>
     <row r="54" spans="1:172" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="17"/>
@@ -11690,11 +11720,11 @@
       <c r="M54" s="20"/>
       <c r="N54" s="20"/>
       <c r="O54" s="20"/>
-      <c r="P54" s="95"/>
+      <c r="P54" s="87"/>
       <c r="Q54" s="88"/>
       <c r="R54" s="88"/>
       <c r="S54" s="89"/>
-      <c r="T54" s="87"/>
+      <c r="T54" s="92"/>
       <c r="U54" s="88"/>
       <c r="V54" s="88"/>
       <c r="W54" s="88"/>
@@ -11730,11 +11760,11 @@
       <c r="BA54" s="20"/>
       <c r="BB54" s="20"/>
       <c r="BC54" s="20"/>
-      <c r="BD54" s="95"/>
+      <c r="BD54" s="87"/>
       <c r="BE54" s="88"/>
       <c r="BF54" s="88"/>
       <c r="BG54" s="89"/>
-      <c r="BH54" s="87"/>
+      <c r="BH54" s="92"/>
       <c r="BI54" s="88"/>
       <c r="BJ54" s="88"/>
       <c r="BK54" s="88"/>
@@ -11742,7 +11772,7 @@
       <c r="BM54" s="88"/>
       <c r="BN54" s="88"/>
       <c r="BO54" s="89"/>
-      <c r="BP54" s="95"/>
+      <c r="BP54" s="87"/>
       <c r="BQ54" s="88"/>
       <c r="BR54" s="88"/>
       <c r="BS54" s="89"/>
@@ -11766,7 +11796,7 @@
       <c r="CK54" s="79"/>
       <c r="CL54" s="79"/>
       <c r="CM54" s="80"/>
-      <c r="CN54" s="87"/>
+      <c r="CN54" s="92"/>
       <c r="CO54" s="88"/>
       <c r="CP54" s="88"/>
       <c r="CQ54" s="88"/>
@@ -11810,11 +11840,11 @@
       <c r="EC54" s="20"/>
       <c r="ED54" s="20"/>
       <c r="EE54" s="20"/>
-      <c r="EF54" s="95"/>
+      <c r="EF54" s="87"/>
       <c r="EG54" s="88"/>
       <c r="EH54" s="88"/>
       <c r="EI54" s="89"/>
-      <c r="EJ54" s="87"/>
+      <c r="EJ54" s="92"/>
       <c r="EK54" s="88"/>
       <c r="EL54" s="88"/>
       <c r="EM54" s="88"/>
@@ -11846,174 +11876,174 @@
       <c r="FM54" s="20"/>
       <c r="FN54" s="20"/>
       <c r="FO54" s="20"/>
-      <c r="FP54" s="101"/>
+      <c r="FP54" s="94"/>
     </row>
     <row r="55" spans="1:172" x14ac:dyDescent="0.2">
-      <c r="A55" s="96" t="s">
+      <c r="A55" s="95" t="s">
         <v>2</v>
       </c>
-      <c r="B55" s="96"/>
-      <c r="C55" s="96"/>
-      <c r="D55" s="96"/>
-      <c r="E55" s="96"/>
-      <c r="F55" s="96"/>
-      <c r="G55" s="96"/>
-      <c r="H55" s="96"/>
-      <c r="I55" s="96"/>
-      <c r="J55" s="96"/>
-      <c r="K55" s="96"/>
-      <c r="L55" s="96"/>
-      <c r="M55" s="96"/>
-      <c r="N55" s="96"/>
-      <c r="O55" s="96"/>
-      <c r="P55" s="96"/>
-      <c r="Q55" s="96"/>
-      <c r="R55" s="96"/>
-      <c r="S55" s="96"/>
-      <c r="T55" s="96"/>
-      <c r="U55" s="96"/>
-      <c r="V55" s="96"/>
-      <c r="W55" s="96"/>
-      <c r="X55" s="96"/>
-      <c r="Y55" s="96"/>
-      <c r="Z55" s="96"/>
-      <c r="AA55" s="96"/>
-      <c r="AB55" s="96"/>
-      <c r="AC55" s="96"/>
-      <c r="AD55" s="96"/>
-      <c r="AE55" s="96"/>
-      <c r="AF55" s="96"/>
-      <c r="AG55" s="96"/>
-      <c r="AH55" s="96"/>
-      <c r="AI55" s="96"/>
-      <c r="AJ55" s="96"/>
-      <c r="AK55" s="96"/>
-      <c r="AL55" s="96"/>
-      <c r="AM55" s="96"/>
-      <c r="AN55" s="96"/>
-      <c r="AO55" s="96"/>
-      <c r="AP55" s="96"/>
-      <c r="AQ55" s="96"/>
-      <c r="AR55" s="96"/>
-      <c r="AS55" s="96"/>
-      <c r="AT55" s="96"/>
-      <c r="AU55" s="96"/>
-      <c r="AV55" s="96"/>
-      <c r="AW55" s="96"/>
-      <c r="AX55" s="96"/>
-      <c r="AY55" s="96"/>
-      <c r="AZ55" s="96"/>
-      <c r="BA55" s="96"/>
-      <c r="BB55" s="96"/>
-      <c r="BC55" s="96"/>
-      <c r="BD55" s="96"/>
-      <c r="BE55" s="96"/>
-      <c r="BF55" s="96"/>
-      <c r="BG55" s="96"/>
-      <c r="BH55" s="96"/>
-      <c r="BI55" s="96"/>
-      <c r="BJ55" s="96"/>
-      <c r="BK55" s="96"/>
-      <c r="BL55" s="96"/>
-      <c r="BM55" s="96"/>
-      <c r="BN55" s="96"/>
-      <c r="BO55" s="96"/>
-      <c r="BP55" s="96"/>
-      <c r="BQ55" s="96"/>
-      <c r="BR55" s="96"/>
-      <c r="BS55" s="96"/>
-      <c r="BT55" s="96"/>
-      <c r="BU55" s="96"/>
-      <c r="BV55" s="96"/>
-      <c r="BW55" s="96"/>
-      <c r="BX55" s="96"/>
-      <c r="BY55" s="96"/>
-      <c r="BZ55" s="96"/>
-      <c r="CA55" s="96"/>
-      <c r="CB55" s="96"/>
-      <c r="CC55" s="96"/>
-      <c r="CD55" s="96"/>
-      <c r="CE55" s="96"/>
-      <c r="CF55" s="96"/>
-      <c r="CG55" s="96"/>
-      <c r="CH55" s="96"/>
-      <c r="CI55" s="96"/>
-      <c r="CJ55" s="96"/>
-      <c r="CK55" s="96"/>
-      <c r="CL55" s="96"/>
-      <c r="CM55" s="96"/>
-      <c r="CN55" s="96"/>
-      <c r="CO55" s="96"/>
-      <c r="CP55" s="96"/>
-      <c r="CQ55" s="96"/>
-      <c r="CR55" s="96"/>
-      <c r="CS55" s="96"/>
-      <c r="CT55" s="96"/>
-      <c r="CU55" s="96"/>
-      <c r="CV55" s="96"/>
-      <c r="CW55" s="96"/>
-      <c r="CX55" s="96"/>
-      <c r="CY55" s="96"/>
-      <c r="CZ55" s="96"/>
-      <c r="DA55" s="96"/>
-      <c r="DB55" s="96"/>
-      <c r="DC55" s="96"/>
-      <c r="DD55" s="96"/>
-      <c r="DE55" s="96"/>
-      <c r="DF55" s="96"/>
-      <c r="DG55" s="96"/>
-      <c r="DH55" s="96"/>
-      <c r="DI55" s="96"/>
-      <c r="DJ55" s="96"/>
-      <c r="DK55" s="96"/>
-      <c r="DL55" s="96"/>
-      <c r="DM55" s="96"/>
-      <c r="DN55" s="96"/>
-      <c r="DO55" s="96"/>
-      <c r="DP55" s="96"/>
-      <c r="DQ55" s="96"/>
-      <c r="DR55" s="96"/>
-      <c r="DS55" s="96"/>
-      <c r="DT55" s="96"/>
-      <c r="DU55" s="96"/>
-      <c r="DV55" s="96"/>
-      <c r="DW55" s="96"/>
-      <c r="DX55" s="96"/>
-      <c r="DY55" s="96"/>
-      <c r="DZ55" s="96"/>
-      <c r="EA55" s="96"/>
-      <c r="EB55" s="96"/>
-      <c r="EC55" s="96"/>
-      <c r="ED55" s="96"/>
-      <c r="EE55" s="96"/>
-      <c r="EF55" s="96"/>
-      <c r="EG55" s="96"/>
-      <c r="EH55" s="96"/>
-      <c r="EI55" s="96"/>
-      <c r="EJ55" s="96"/>
-      <c r="EK55" s="96"/>
-      <c r="EL55" s="96"/>
-      <c r="EM55" s="96"/>
-      <c r="EN55" s="96"/>
-      <c r="EO55" s="96"/>
-      <c r="EP55" s="96"/>
-      <c r="EQ55" s="96"/>
-      <c r="ER55" s="96"/>
-      <c r="ES55" s="96"/>
-      <c r="ET55" s="96"/>
-      <c r="EU55" s="96"/>
-      <c r="EV55" s="96"/>
-      <c r="EW55" s="96"/>
-      <c r="EX55" s="96"/>
-      <c r="EY55" s="96"/>
-      <c r="EZ55" s="96"/>
-      <c r="FA55" s="96"/>
-      <c r="FB55" s="96"/>
-      <c r="FC55" s="96"/>
-      <c r="FD55" s="96"/>
-      <c r="FE55" s="96"/>
-      <c r="FF55" s="96"/>
-      <c r="FG55" s="96"/>
+      <c r="B55" s="95"/>
+      <c r="C55" s="95"/>
+      <c r="D55" s="95"/>
+      <c r="E55" s="95"/>
+      <c r="F55" s="95"/>
+      <c r="G55" s="95"/>
+      <c r="H55" s="95"/>
+      <c r="I55" s="95"/>
+      <c r="J55" s="95"/>
+      <c r="K55" s="95"/>
+      <c r="L55" s="95"/>
+      <c r="M55" s="95"/>
+      <c r="N55" s="95"/>
+      <c r="O55" s="95"/>
+      <c r="P55" s="95"/>
+      <c r="Q55" s="95"/>
+      <c r="R55" s="95"/>
+      <c r="S55" s="95"/>
+      <c r="T55" s="95"/>
+      <c r="U55" s="95"/>
+      <c r="V55" s="95"/>
+      <c r="W55" s="95"/>
+      <c r="X55" s="95"/>
+      <c r="Y55" s="95"/>
+      <c r="Z55" s="95"/>
+      <c r="AA55" s="95"/>
+      <c r="AB55" s="95"/>
+      <c r="AC55" s="95"/>
+      <c r="AD55" s="95"/>
+      <c r="AE55" s="95"/>
+      <c r="AF55" s="95"/>
+      <c r="AG55" s="95"/>
+      <c r="AH55" s="95"/>
+      <c r="AI55" s="95"/>
+      <c r="AJ55" s="95"/>
+      <c r="AK55" s="95"/>
+      <c r="AL55" s="95"/>
+      <c r="AM55" s="95"/>
+      <c r="AN55" s="95"/>
+      <c r="AO55" s="95"/>
+      <c r="AP55" s="95"/>
+      <c r="AQ55" s="95"/>
+      <c r="AR55" s="95"/>
+      <c r="AS55" s="95"/>
+      <c r="AT55" s="95"/>
+      <c r="AU55" s="95"/>
+      <c r="AV55" s="95"/>
+      <c r="AW55" s="95"/>
+      <c r="AX55" s="95"/>
+      <c r="AY55" s="95"/>
+      <c r="AZ55" s="95"/>
+      <c r="BA55" s="95"/>
+      <c r="BB55" s="95"/>
+      <c r="BC55" s="95"/>
+      <c r="BD55" s="95"/>
+      <c r="BE55" s="95"/>
+      <c r="BF55" s="95"/>
+      <c r="BG55" s="95"/>
+      <c r="BH55" s="95"/>
+      <c r="BI55" s="95"/>
+      <c r="BJ55" s="95"/>
+      <c r="BK55" s="95"/>
+      <c r="BL55" s="95"/>
+      <c r="BM55" s="95"/>
+      <c r="BN55" s="95"/>
+      <c r="BO55" s="95"/>
+      <c r="BP55" s="95"/>
+      <c r="BQ55" s="95"/>
+      <c r="BR55" s="95"/>
+      <c r="BS55" s="95"/>
+      <c r="BT55" s="95"/>
+      <c r="BU55" s="95"/>
+      <c r="BV55" s="95"/>
+      <c r="BW55" s="95"/>
+      <c r="BX55" s="95"/>
+      <c r="BY55" s="95"/>
+      <c r="BZ55" s="95"/>
+      <c r="CA55" s="95"/>
+      <c r="CB55" s="95"/>
+      <c r="CC55" s="95"/>
+      <c r="CD55" s="95"/>
+      <c r="CE55" s="95"/>
+      <c r="CF55" s="95"/>
+      <c r="CG55" s="95"/>
+      <c r="CH55" s="95"/>
+      <c r="CI55" s="95"/>
+      <c r="CJ55" s="95"/>
+      <c r="CK55" s="95"/>
+      <c r="CL55" s="95"/>
+      <c r="CM55" s="95"/>
+      <c r="CN55" s="95"/>
+      <c r="CO55" s="95"/>
+      <c r="CP55" s="95"/>
+      <c r="CQ55" s="95"/>
+      <c r="CR55" s="95"/>
+      <c r="CS55" s="95"/>
+      <c r="CT55" s="95"/>
+      <c r="CU55" s="95"/>
+      <c r="CV55" s="95"/>
+      <c r="CW55" s="95"/>
+      <c r="CX55" s="95"/>
+      <c r="CY55" s="95"/>
+      <c r="CZ55" s="95"/>
+      <c r="DA55" s="95"/>
+      <c r="DB55" s="95"/>
+      <c r="DC55" s="95"/>
+      <c r="DD55" s="95"/>
+      <c r="DE55" s="95"/>
+      <c r="DF55" s="95"/>
+      <c r="DG55" s="95"/>
+      <c r="DH55" s="95"/>
+      <c r="DI55" s="95"/>
+      <c r="DJ55" s="95"/>
+      <c r="DK55" s="95"/>
+      <c r="DL55" s="95"/>
+      <c r="DM55" s="95"/>
+      <c r="DN55" s="95"/>
+      <c r="DO55" s="95"/>
+      <c r="DP55" s="95"/>
+      <c r="DQ55" s="95"/>
+      <c r="DR55" s="95"/>
+      <c r="DS55" s="95"/>
+      <c r="DT55" s="95"/>
+      <c r="DU55" s="95"/>
+      <c r="DV55" s="95"/>
+      <c r="DW55" s="95"/>
+      <c r="DX55" s="95"/>
+      <c r="DY55" s="95"/>
+      <c r="DZ55" s="95"/>
+      <c r="EA55" s="95"/>
+      <c r="EB55" s="95"/>
+      <c r="EC55" s="95"/>
+      <c r="ED55" s="95"/>
+      <c r="EE55" s="95"/>
+      <c r="EF55" s="95"/>
+      <c r="EG55" s="95"/>
+      <c r="EH55" s="95"/>
+      <c r="EI55" s="95"/>
+      <c r="EJ55" s="95"/>
+      <c r="EK55" s="95"/>
+      <c r="EL55" s="95"/>
+      <c r="EM55" s="95"/>
+      <c r="EN55" s="95"/>
+      <c r="EO55" s="95"/>
+      <c r="EP55" s="95"/>
+      <c r="EQ55" s="95"/>
+      <c r="ER55" s="95"/>
+      <c r="ES55" s="95"/>
+      <c r="ET55" s="95"/>
+      <c r="EU55" s="95"/>
+      <c r="EV55" s="95"/>
+      <c r="EW55" s="95"/>
+      <c r="EX55" s="95"/>
+      <c r="EY55" s="95"/>
+      <c r="EZ55" s="95"/>
+      <c r="FA55" s="95"/>
+      <c r="FB55" s="95"/>
+      <c r="FC55" s="95"/>
+      <c r="FD55" s="95"/>
+      <c r="FE55" s="95"/>
+      <c r="FF55" s="95"/>
+      <c r="FG55" s="95"/>
       <c r="FH55" s="38"/>
       <c r="FI55" s="38"/>
       <c r="FJ55" s="38"/>
@@ -12025,24 +12055,34 @@
     </row>
   </sheetData>
   <mergeCells count="62">
-    <mergeCell ref="AN4:AQ4"/>
-    <mergeCell ref="AR4:AU4"/>
-    <mergeCell ref="CZ4:DC4"/>
-    <mergeCell ref="CF6:CM54"/>
-    <mergeCell ref="BD6:BG54"/>
-    <mergeCell ref="BH6:BO54"/>
-    <mergeCell ref="CN6:DK54"/>
-    <mergeCell ref="FP4:FP54"/>
-    <mergeCell ref="EJ4:EM4"/>
-    <mergeCell ref="EN4:EQ4"/>
-    <mergeCell ref="ER4:EU4"/>
-    <mergeCell ref="EV4:EY4"/>
-    <mergeCell ref="EZ4:FC4"/>
-    <mergeCell ref="FD4:FG4"/>
-    <mergeCell ref="ER6:EY54"/>
-    <mergeCell ref="EJ6:EQ54"/>
-    <mergeCell ref="FL4:FO4"/>
-    <mergeCell ref="FH4:FK4"/>
+    <mergeCell ref="DP4:DS4"/>
+    <mergeCell ref="AV4:AY4"/>
+    <mergeCell ref="AZ4:BC4"/>
+    <mergeCell ref="BL4:BO4"/>
+    <mergeCell ref="BH4:BK4"/>
+    <mergeCell ref="CF4:CI4"/>
+    <mergeCell ref="CJ4:CM4"/>
+    <mergeCell ref="CN4:CQ4"/>
+    <mergeCell ref="CR4:CU4"/>
+    <mergeCell ref="DH4:DK4"/>
+    <mergeCell ref="DL4:DO4"/>
+    <mergeCell ref="CB4:CE4"/>
+    <mergeCell ref="BT4:BW4"/>
+    <mergeCell ref="DD4:DG4"/>
+    <mergeCell ref="BP4:BS4"/>
+    <mergeCell ref="AJ4:AM4"/>
+    <mergeCell ref="AB6:AI54"/>
+    <mergeCell ref="T6:AA54"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D4:G4"/>
+    <mergeCell ref="H4:K4"/>
+    <mergeCell ref="P6:S54"/>
+    <mergeCell ref="P4:S4"/>
+    <mergeCell ref="T4:W4"/>
+    <mergeCell ref="X4:AA4"/>
+    <mergeCell ref="AB4:AE4"/>
+    <mergeCell ref="AF4:AI4"/>
     <mergeCell ref="A55:FG55"/>
     <mergeCell ref="A4:A5"/>
     <mergeCell ref="CF2:DS3"/>
@@ -12059,34 +12099,24 @@
     <mergeCell ref="EF6:EI54"/>
     <mergeCell ref="L4:O4"/>
     <mergeCell ref="BP6:BS54"/>
-    <mergeCell ref="AJ4:AM4"/>
-    <mergeCell ref="AB6:AI54"/>
-    <mergeCell ref="T6:AA54"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D4:G4"/>
-    <mergeCell ref="H4:K4"/>
-    <mergeCell ref="P6:S54"/>
-    <mergeCell ref="P4:S4"/>
-    <mergeCell ref="T4:W4"/>
-    <mergeCell ref="X4:AA4"/>
-    <mergeCell ref="AB4:AE4"/>
-    <mergeCell ref="AF4:AI4"/>
-    <mergeCell ref="DP4:DS4"/>
-    <mergeCell ref="AV4:AY4"/>
-    <mergeCell ref="AZ4:BC4"/>
-    <mergeCell ref="BL4:BO4"/>
-    <mergeCell ref="BH4:BK4"/>
-    <mergeCell ref="CF4:CI4"/>
-    <mergeCell ref="CJ4:CM4"/>
-    <mergeCell ref="CN4:CQ4"/>
-    <mergeCell ref="CR4:CU4"/>
-    <mergeCell ref="DH4:DK4"/>
-    <mergeCell ref="DL4:DO4"/>
-    <mergeCell ref="CB4:CE4"/>
-    <mergeCell ref="BT4:BW4"/>
-    <mergeCell ref="DD4:DG4"/>
-    <mergeCell ref="BP4:BS4"/>
+    <mergeCell ref="FP4:FP54"/>
+    <mergeCell ref="EJ4:EM4"/>
+    <mergeCell ref="EN4:EQ4"/>
+    <mergeCell ref="ER4:EU4"/>
+    <mergeCell ref="EV4:EY4"/>
+    <mergeCell ref="EZ4:FC4"/>
+    <mergeCell ref="FD4:FG4"/>
+    <mergeCell ref="ER6:EY54"/>
+    <mergeCell ref="EJ6:EQ54"/>
+    <mergeCell ref="FL4:FO4"/>
+    <mergeCell ref="FH4:FK4"/>
+    <mergeCell ref="AN4:AQ4"/>
+    <mergeCell ref="AR4:AU4"/>
+    <mergeCell ref="CZ4:DC4"/>
+    <mergeCell ref="CF6:CM54"/>
+    <mergeCell ref="BD6:BG54"/>
+    <mergeCell ref="BH6:BO54"/>
+    <mergeCell ref="CN6:DK54"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B54">
     <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Terminé">

</xml_diff>